<commit_message>
Revise staffing plan from updated assignments
- Toyo Nassen RD: Kawate + Sakuma (Kozono off)
- Yutaka Shoji Dev: 6 -> 4 MM
- Iwatani Dev: add Ito
- Recalculate per-person monthly load; Kawate remains Oct-Dec bottleneck

Co-authored-by: kozonoflight <kozonoflight@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/knowledge/人積み/2026-2027_案件人積み.xlsx
+++ b/knowledge/人積み/2026-2027_案件人積み.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet name="人積み一覧" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'人積み一覧'!$1:$11</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -94,7 +92,7 @@
       <sz val="7"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -168,7 +166,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00E8DFF5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00D9E2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0020B2AA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="009B7EBD"/>
       </patternFill>
     </fill>
   </fills>
@@ -198,7 +211,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -233,8 +246,11 @@
     <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -260,46 +276,52 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -667,19 +689,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X62"/>
+  <dimension ref="A1:X64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="5.8" customWidth="1" min="7" max="7"/>
     <col width="5.8" customWidth="1" min="8" max="8"/>
     <col width="5.8" customWidth="1" min="9" max="9"/>
-    <col width="5.8" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
     <col width="5.8" customWidth="1" min="11" max="11"/>
     <col width="5.8" customWidth="1" min="12" max="12"/>
     <col width="5.8" customWidth="1" min="13" max="13"/>
@@ -699,21 +721,21 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>案件人積み・スケジュール俯瞰（1シート完結）</t>
+          <t>案件人積み・スケジュール俯瞰（1シート完結）※割当見直し反映</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>前提: 今期=26/4〜27/3・来期=27/4〜。工数は期間均等按分。灰セル=?時期未定だが工数は判明 → セル内に人月を記載。</t>
+          <t>更新: 豊商事Dev=4人月 / 東洋捺染RD=川手・佐久間 / イワタニDev=木村・森崎（伊藤）。負荷は担当者別に再計算（工数は担当人数で按分）。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>① 一目サマリ</t>
+          <t>① 一目サマリ（見直し後）</t>
         </is>
       </c>
     </row>
@@ -725,45 +747,45 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>26/10〜12：川手・小園のRDが最大3件同時（イシダ・三菱・東洋捺染）。キャパ2.0に対し負荷≈3.7</t>
+          <t>26/10〜12：川手が3案件同時（イシダ・三菱・東洋捺染）で月≈1.8人月超。小園は東洋から外れ≈1.2まで改善も、イシダ+三菱でなお逼迫</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>成立帯</t>
+          <t>改善点</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>26/8〜9：ローリングスRD（川手・小園）＋イワタニDev（木村・森崎）</t>
+          <t>東洋捺染RDに佐久間を投入 → 小園の10〜12月負荷が軽減。豊商事Dev 6→4人月で未割当Dev合計≈111.35</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>未割当</t>
+          <t>残課題</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>開発の大半が未割当（合計≈112人月）。東洋捺染≈40が突出。灰帯は時期未定でも工数あり</t>
+          <t>開発の大半が未割当。ローリングスDev・豊商事・イシダDevの担当決めが必要。神鋼・アムリードは時期未定の隠し負荷</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>② 簡易ガント（これだけ見ればスケジュールと工数が分かる）</t>
+          <t>② 簡易ガント</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>凡例: R=要件定義(青) / D=開発・担当あり(緑) / U=開発・未割当(黄) / 数字のみの灰=?時期未定だが工数判明（人月） / 黄列ヘッダ=来期</t>
+          <t>凡例: R=要件定義 / D=開発・担当あり / U=開発・未割当 / 灰+数字=時期未定だが工数判明 / 黄列ヘッダ=来期</t>
         </is>
       </c>
     </row>
@@ -898,7 +920,7 @@
       <c r="B12" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>川手・小園</t>
         </is>
@@ -906,120 +928,120 @@
       <c r="D12" s="13" t="n">
         <v>4.5</v>
       </c>
-      <c r="E12" s="14" t="inlineStr">
+      <c r="E12" s="15" t="inlineStr">
         <is>
           <t>未割当</t>
         </is>
       </c>
-      <c r="F12" s="15" t="inlineStr">
-        <is>
-          <t>10月重複</t>
-        </is>
-      </c>
-      <c r="G12" s="16" t="inlineStr"/>
-      <c r="H12" s="16" t="inlineStr"/>
-      <c r="I12" s="17" t="inlineStr">
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>重複</t>
+        </is>
+      </c>
+      <c r="G12" s="17" t="inlineStr"/>
+      <c r="H12" s="17" t="inlineStr"/>
+      <c r="I12" s="18" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="J12" s="17" t="inlineStr">
+      <c r="J12" s="18" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="K12" s="16" t="inlineStr"/>
-      <c r="L12" s="18" t="inlineStr">
+      <c r="K12" s="17" t="inlineStr"/>
+      <c r="L12" s="19" t="inlineStr">
         <is>
           <t>U4.5</t>
         </is>
       </c>
-      <c r="M12" s="18" t="inlineStr">
+      <c r="M12" s="19" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="N12" s="18" t="inlineStr">
+      <c r="N12" s="19" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="O12" s="19" t="inlineStr"/>
-      <c r="P12" s="19" t="inlineStr"/>
-      <c r="Q12" s="19" t="inlineStr"/>
-      <c r="R12" s="19" t="inlineStr"/>
-      <c r="S12" s="19" t="inlineStr"/>
-      <c r="T12" s="19" t="inlineStr"/>
-      <c r="U12" s="19" t="inlineStr"/>
-      <c r="V12" s="19" t="inlineStr"/>
-      <c r="W12" s="19" t="inlineStr"/>
-      <c r="X12" s="19" t="inlineStr"/>
+      <c r="O12" s="20" t="inlineStr"/>
+      <c r="P12" s="20" t="inlineStr"/>
+      <c r="Q12" s="20" t="inlineStr"/>
+      <c r="R12" s="20" t="inlineStr"/>
+      <c r="S12" s="20" t="inlineStr"/>
+      <c r="T12" s="20" t="inlineStr"/>
+      <c r="U12" s="20" t="inlineStr"/>
+      <c r="V12" s="20" t="inlineStr"/>
+      <c r="W12" s="20" t="inlineStr"/>
+      <c r="X12" s="20" t="inlineStr"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="20" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>ローリングスジャパン</t>
         </is>
       </c>
-      <c r="B13" s="21" t="n">
+      <c r="B13" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="21" t="inlineStr">
+      <c r="C13" s="23" t="inlineStr">
         <is>
           <t>川手・小園</t>
         </is>
       </c>
-      <c r="D13" s="21" t="n">
+      <c r="D13" s="22" t="n">
         <v>4.4</v>
       </c>
-      <c r="E13" s="14" t="inlineStr">
+      <c r="E13" s="15" t="inlineStr">
         <is>
           <t>未割当</t>
         </is>
       </c>
-      <c r="F13" s="22" t="inlineStr">
+      <c r="F13" s="23" t="inlineStr">
         <is>
           <t>Devは別担当必須</t>
         </is>
       </c>
-      <c r="G13" s="17" t="inlineStr">
+      <c r="G13" s="18" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="H13" s="17" t="inlineStr">
+      <c r="H13" s="18" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="I13" s="18" t="inlineStr">
+      <c r="I13" s="19" t="inlineStr">
         <is>
           <t>U4.4</t>
         </is>
       </c>
-      <c r="J13" s="18" t="inlineStr">
+      <c r="J13" s="19" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="K13" s="18" t="inlineStr">
+      <c r="K13" s="19" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="L13" s="16" t="inlineStr"/>
-      <c r="M13" s="16" t="inlineStr"/>
-      <c r="N13" s="16" t="inlineStr"/>
-      <c r="O13" s="19" t="inlineStr"/>
-      <c r="P13" s="19" t="inlineStr"/>
-      <c r="Q13" s="19" t="inlineStr"/>
-      <c r="R13" s="19" t="inlineStr"/>
-      <c r="S13" s="19" t="inlineStr"/>
-      <c r="T13" s="19" t="inlineStr"/>
-      <c r="U13" s="19" t="inlineStr"/>
-      <c r="V13" s="19" t="inlineStr"/>
-      <c r="W13" s="19" t="inlineStr"/>
-      <c r="X13" s="19" t="inlineStr"/>
+      <c r="L13" s="17" t="inlineStr"/>
+      <c r="M13" s="17" t="inlineStr"/>
+      <c r="N13" s="17" t="inlineStr"/>
+      <c r="O13" s="20" t="inlineStr"/>
+      <c r="P13" s="20" t="inlineStr"/>
+      <c r="Q13" s="20" t="inlineStr"/>
+      <c r="R13" s="20" t="inlineStr"/>
+      <c r="S13" s="20" t="inlineStr"/>
+      <c r="T13" s="20" t="inlineStr"/>
+      <c r="U13" s="20" t="inlineStr"/>
+      <c r="V13" s="20" t="inlineStr"/>
+      <c r="W13" s="20" t="inlineStr"/>
+      <c r="X13" s="20" t="inlineStr"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="12" t="inlineStr">
@@ -1032,7 +1054,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1040,12 +1062,12 @@
       <c r="D14" s="13" t="n">
         <v>1.5</v>
       </c>
-      <c r="E14" s="13" t="inlineStr">
-        <is>
-          <t>木村・森崎</t>
-        </is>
-      </c>
-      <c r="F14" s="23" t="inlineStr">
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>木村・森崎（伊藤）</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
         <is>
           <t>成立</t>
         </is>
@@ -1060,86 +1082,86 @@
           <t>D</t>
         </is>
       </c>
-      <c r="I14" s="16" t="inlineStr"/>
-      <c r="J14" s="16" t="inlineStr"/>
-      <c r="K14" s="16" t="inlineStr"/>
-      <c r="L14" s="16" t="inlineStr"/>
-      <c r="M14" s="16" t="inlineStr"/>
-      <c r="N14" s="16" t="inlineStr"/>
-      <c r="O14" s="19" t="inlineStr"/>
-      <c r="P14" s="19" t="inlineStr"/>
-      <c r="Q14" s="19" t="inlineStr"/>
-      <c r="R14" s="19" t="inlineStr"/>
-      <c r="S14" s="19" t="inlineStr"/>
-      <c r="T14" s="19" t="inlineStr"/>
-      <c r="U14" s="19" t="inlineStr"/>
-      <c r="V14" s="19" t="inlineStr"/>
-      <c r="W14" s="19" t="inlineStr"/>
-      <c r="X14" s="19" t="inlineStr"/>
+      <c r="I14" s="17" t="inlineStr"/>
+      <c r="J14" s="17" t="inlineStr"/>
+      <c r="K14" s="17" t="inlineStr"/>
+      <c r="L14" s="17" t="inlineStr"/>
+      <c r="M14" s="17" t="inlineStr"/>
+      <c r="N14" s="17" t="inlineStr"/>
+      <c r="O14" s="20" t="inlineStr"/>
+      <c r="P14" s="20" t="inlineStr"/>
+      <c r="Q14" s="20" t="inlineStr"/>
+      <c r="R14" s="20" t="inlineStr"/>
+      <c r="S14" s="20" t="inlineStr"/>
+      <c r="T14" s="20" t="inlineStr"/>
+      <c r="U14" s="20" t="inlineStr"/>
+      <c r="V14" s="20" t="inlineStr"/>
+      <c r="W14" s="20" t="inlineStr"/>
+      <c r="X14" s="20" t="inlineStr"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="20" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>豊商事</t>
         </is>
       </c>
-      <c r="B15" s="21" t="inlineStr">
+      <c r="B15" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C15" s="21" t="inlineStr">
+      <c r="C15" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D15" s="21" t="n">
-        <v>6</v>
-      </c>
-      <c r="E15" s="14" t="inlineStr">
+      <c r="D15" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
         <is>
           <t>未割当</t>
         </is>
       </c>
-      <c r="F15" s="22" t="inlineStr">
+      <c r="F15" s="16" t="inlineStr">
         <is>
           <t>時期仮・RD帯と重複</t>
         </is>
       </c>
-      <c r="G15" s="16" t="inlineStr"/>
-      <c r="H15" s="18" t="inlineStr">
-        <is>
-          <t>U≈6</t>
-        </is>
-      </c>
-      <c r="I15" s="18" t="inlineStr">
+      <c r="G15" s="17" t="inlineStr"/>
+      <c r="H15" s="19" t="inlineStr">
+        <is>
+          <t>U≈4</t>
+        </is>
+      </c>
+      <c r="I15" s="19" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="J15" s="18" t="inlineStr">
+      <c r="J15" s="19" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="K15" s="18" t="inlineStr">
+      <c r="K15" s="19" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="L15" s="16" t="inlineStr"/>
-      <c r="M15" s="16" t="inlineStr"/>
-      <c r="N15" s="16" t="inlineStr"/>
-      <c r="O15" s="19" t="inlineStr"/>
-      <c r="P15" s="19" t="inlineStr"/>
-      <c r="Q15" s="19" t="inlineStr"/>
-      <c r="R15" s="19" t="inlineStr"/>
-      <c r="S15" s="19" t="inlineStr"/>
-      <c r="T15" s="19" t="inlineStr"/>
-      <c r="U15" s="19" t="inlineStr"/>
-      <c r="V15" s="19" t="inlineStr"/>
-      <c r="W15" s="19" t="inlineStr"/>
-      <c r="X15" s="19" t="inlineStr"/>
+      <c r="L15" s="17" t="inlineStr"/>
+      <c r="M15" s="17" t="inlineStr"/>
+      <c r="N15" s="17" t="inlineStr"/>
+      <c r="O15" s="20" t="inlineStr"/>
+      <c r="P15" s="20" t="inlineStr"/>
+      <c r="Q15" s="20" t="inlineStr"/>
+      <c r="R15" s="20" t="inlineStr"/>
+      <c r="S15" s="20" t="inlineStr"/>
+      <c r="T15" s="20" t="inlineStr"/>
+      <c r="U15" s="20" t="inlineStr"/>
+      <c r="V15" s="20" t="inlineStr"/>
+      <c r="W15" s="20" t="inlineStr"/>
+      <c r="X15" s="20" t="inlineStr"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="12" t="inlineStr">
@@ -1150,7 +1172,7 @@
       <c r="B16" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>川手・小園</t>
         </is>
@@ -1158,36 +1180,36 @@
       <c r="D16" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="E16" s="14" t="inlineStr">
+      <c r="E16" s="15" t="inlineStr">
         <is>
           <t>未割当</t>
         </is>
       </c>
-      <c r="F16" s="15" t="inlineStr">
-        <is>
-          <t>RDスライド候補</t>
-        </is>
-      </c>
-      <c r="G16" s="16" t="inlineStr"/>
-      <c r="H16" s="16" t="inlineStr"/>
-      <c r="I16" s="17" t="inlineStr">
+      <c r="F16" s="16" t="inlineStr">
+        <is>
+          <t>重複・スライド候補</t>
+        </is>
+      </c>
+      <c r="G16" s="17" t="inlineStr"/>
+      <c r="H16" s="17" t="inlineStr"/>
+      <c r="I16" s="18" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="J16" s="17" t="inlineStr">
+      <c r="J16" s="18" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="K16" s="17" t="inlineStr">
+      <c r="K16" s="18" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="L16" s="16" t="inlineStr"/>
-      <c r="M16" s="16" t="inlineStr"/>
-      <c r="N16" s="16" t="inlineStr"/>
+      <c r="L16" s="17" t="inlineStr"/>
+      <c r="M16" s="17" t="inlineStr"/>
+      <c r="N16" s="17" t="inlineStr"/>
       <c r="O16" s="25" t="inlineStr">
         <is>
           <t>≈10人月</t>
@@ -1240,52 +1262,52 @@
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>東洋捺染</t>
         </is>
       </c>
-      <c r="B17" s="21" t="n">
+      <c r="B17" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="C17" s="21" t="inlineStr">
-        <is>
-          <t>川手・小園</t>
-        </is>
-      </c>
-      <c r="D17" s="21" t="n">
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>川手・佐久間</t>
+        </is>
+      </c>
+      <c r="D17" s="22" t="n">
         <v>40</v>
       </c>
-      <c r="E17" s="14" t="inlineStr">
+      <c r="E17" s="15" t="inlineStr">
         <is>
           <t>未割当</t>
         </is>
       </c>
-      <c r="F17" s="15" t="inlineStr">
-        <is>
-          <t>大型・専用チーム検討</t>
-        </is>
-      </c>
-      <c r="G17" s="16" t="inlineStr"/>
-      <c r="H17" s="16" t="inlineStr"/>
-      <c r="I17" s="17" t="inlineStr">
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>重複・大型</t>
+        </is>
+      </c>
+      <c r="G17" s="17" t="inlineStr"/>
+      <c r="H17" s="17" t="inlineStr"/>
+      <c r="I17" s="18" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="J17" s="17" t="inlineStr">
+      <c r="J17" s="18" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="K17" s="17" t="inlineStr">
+      <c r="K17" s="18" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="L17" s="16" t="inlineStr"/>
-      <c r="M17" s="16" t="inlineStr"/>
-      <c r="N17" s="16" t="inlineStr"/>
+      <c r="L17" s="17" t="inlineStr"/>
+      <c r="M17" s="17" t="inlineStr"/>
+      <c r="N17" s="17" t="inlineStr"/>
       <c r="O17" s="25" t="inlineStr">
         <is>
           <t>≈40人月</t>
@@ -1346,7 +1368,7 @@
       <c r="B18" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="C18" s="13" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>川手</t>
         </is>
@@ -1354,12 +1376,12 @@
       <c r="D18" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="E18" s="14" t="inlineStr">
+      <c r="E18" s="15" t="inlineStr">
         <is>
           <t>未割当</t>
         </is>
       </c>
-      <c r="F18" s="23" t="inlineStr">
+      <c r="F18" s="14" t="inlineStr">
         <is>
           <t>今期？時期未定</t>
         </is>
@@ -1404,42 +1426,42 @@
           <t>…</t>
         </is>
       </c>
-      <c r="O18" s="19" t="inlineStr"/>
-      <c r="P18" s="19" t="inlineStr"/>
-      <c r="Q18" s="19" t="inlineStr"/>
-      <c r="R18" s="19" t="inlineStr"/>
-      <c r="S18" s="19" t="inlineStr"/>
-      <c r="T18" s="19" t="inlineStr"/>
-      <c r="U18" s="19" t="inlineStr"/>
-      <c r="V18" s="19" t="inlineStr"/>
-      <c r="W18" s="19" t="inlineStr"/>
-      <c r="X18" s="19" t="inlineStr"/>
+      <c r="O18" s="20" t="inlineStr"/>
+      <c r="P18" s="20" t="inlineStr"/>
+      <c r="Q18" s="20" t="inlineStr"/>
+      <c r="R18" s="20" t="inlineStr"/>
+      <c r="S18" s="20" t="inlineStr"/>
+      <c r="T18" s="20" t="inlineStr"/>
+      <c r="U18" s="20" t="inlineStr"/>
+      <c r="V18" s="20" t="inlineStr"/>
+      <c r="W18" s="20" t="inlineStr"/>
+      <c r="X18" s="20" t="inlineStr"/>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="20" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>アムリード</t>
         </is>
       </c>
-      <c r="B19" s="21" t="n">
+      <c r="B19" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="C19" s="21" t="inlineStr">
+      <c r="C19" s="23" t="inlineStr">
         <is>
           <t>川手・小園</t>
         </is>
       </c>
-      <c r="D19" s="21" t="n">
+      <c r="D19" s="22" t="n">
         <v>1.5</v>
       </c>
-      <c r="E19" s="14" t="inlineStr">
+      <c r="E19" s="15" t="inlineStr">
         <is>
           <t>未割当</t>
         </is>
       </c>
-      <c r="F19" s="15" t="inlineStr">
-        <is>
-          <t>時期不明・隠し負荷</t>
+      <c r="F19" s="23" t="inlineStr">
+        <is>
+          <t>時期未定</t>
         </is>
       </c>
       <c r="G19" s="25" t="inlineStr">
@@ -1482,16 +1504,16 @@
           <t>…</t>
         </is>
       </c>
-      <c r="O19" s="19" t="inlineStr"/>
-      <c r="P19" s="19" t="inlineStr"/>
-      <c r="Q19" s="19" t="inlineStr"/>
-      <c r="R19" s="19" t="inlineStr"/>
-      <c r="S19" s="19" t="inlineStr"/>
-      <c r="T19" s="19" t="inlineStr"/>
-      <c r="U19" s="19" t="inlineStr"/>
-      <c r="V19" s="19" t="inlineStr"/>
-      <c r="W19" s="19" t="inlineStr"/>
-      <c r="X19" s="19" t="inlineStr"/>
+      <c r="O19" s="20" t="inlineStr"/>
+      <c r="P19" s="20" t="inlineStr"/>
+      <c r="Q19" s="20" t="inlineStr"/>
+      <c r="R19" s="20" t="inlineStr"/>
+      <c r="S19" s="20" t="inlineStr"/>
+      <c r="T19" s="20" t="inlineStr"/>
+      <c r="U19" s="20" t="inlineStr"/>
+      <c r="V19" s="20" t="inlineStr"/>
+      <c r="W19" s="20" t="inlineStr"/>
+      <c r="X19" s="20" t="inlineStr"/>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="12" t="inlineStr">
@@ -1502,7 +1524,7 @@
       <c r="B20" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="C20" s="13" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr">
         <is>
           <t>川手・小園</t>
         </is>
@@ -1510,24 +1532,24 @@
       <c r="D20" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="E20" s="14" t="inlineStr">
+      <c r="E20" s="15" t="inlineStr">
         <is>
           <t>未割当</t>
         </is>
       </c>
-      <c r="F20" s="23" t="inlineStr">
-        <is>
-          <t>来期・スロット化</t>
-        </is>
-      </c>
-      <c r="G20" s="16" t="inlineStr"/>
-      <c r="H20" s="16" t="inlineStr"/>
-      <c r="I20" s="16" t="inlineStr"/>
-      <c r="J20" s="16" t="inlineStr"/>
-      <c r="K20" s="16" t="inlineStr"/>
-      <c r="L20" s="16" t="inlineStr"/>
-      <c r="M20" s="16" t="inlineStr"/>
-      <c r="N20" s="16" t="inlineStr"/>
+      <c r="F20" s="14" t="inlineStr">
+        <is>
+          <t>来期</t>
+        </is>
+      </c>
+      <c r="G20" s="17" t="inlineStr"/>
+      <c r="H20" s="17" t="inlineStr"/>
+      <c r="I20" s="17" t="inlineStr"/>
+      <c r="J20" s="17" t="inlineStr"/>
+      <c r="K20" s="17" t="inlineStr"/>
+      <c r="L20" s="17" t="inlineStr"/>
+      <c r="M20" s="17" t="inlineStr"/>
+      <c r="N20" s="17" t="inlineStr"/>
       <c r="O20" s="25" t="inlineStr">
         <is>
           <t>RD3+Dev10</t>
@@ -1580,42 +1602,42 @@
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="20" t="inlineStr">
+      <c r="A21" s="21" t="inlineStr">
         <is>
           <t>日東電工BM</t>
         </is>
       </c>
-      <c r="B21" s="21" t="inlineStr">
+      <c r="B21" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C21" s="21" t="inlineStr">
+      <c r="C21" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D21" s="21" t="n">
+      <c r="D21" s="22" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E21" s="15" t="inlineStr">
         <is>
           <t>未割当</t>
         </is>
       </c>
-      <c r="F21" s="22" t="inlineStr">
+      <c r="F21" s="23" t="inlineStr">
         <is>
           <t>来期</t>
         </is>
       </c>
-      <c r="G21" s="16" t="inlineStr"/>
-      <c r="H21" s="16" t="inlineStr"/>
-      <c r="I21" s="16" t="inlineStr"/>
-      <c r="J21" s="16" t="inlineStr"/>
-      <c r="K21" s="16" t="inlineStr"/>
-      <c r="L21" s="16" t="inlineStr"/>
-      <c r="M21" s="16" t="inlineStr"/>
-      <c r="N21" s="16" t="inlineStr"/>
+      <c r="G21" s="17" t="inlineStr"/>
+      <c r="H21" s="17" t="inlineStr"/>
+      <c r="I21" s="17" t="inlineStr"/>
+      <c r="J21" s="17" t="inlineStr"/>
+      <c r="K21" s="17" t="inlineStr"/>
+      <c r="L21" s="17" t="inlineStr"/>
+      <c r="M21" s="17" t="inlineStr"/>
+      <c r="N21" s="17" t="inlineStr"/>
       <c r="O21" s="25" t="inlineStr">
         <is>
           <t>≈8.8人月</t>
@@ -1678,7 +1700,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C22" s="13" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1686,24 +1708,24 @@
       <c r="D22" s="13" t="n">
         <v>8.6</v>
       </c>
-      <c r="E22" s="14" t="inlineStr">
+      <c r="E22" s="15" t="inlineStr">
         <is>
           <t>未割当</t>
         </is>
       </c>
-      <c r="F22" s="23" t="inlineStr">
+      <c r="F22" s="14" t="inlineStr">
         <is>
           <t>来期</t>
         </is>
       </c>
-      <c r="G22" s="16" t="inlineStr"/>
-      <c r="H22" s="16" t="inlineStr"/>
-      <c r="I22" s="16" t="inlineStr"/>
-      <c r="J22" s="16" t="inlineStr"/>
-      <c r="K22" s="16" t="inlineStr"/>
-      <c r="L22" s="16" t="inlineStr"/>
-      <c r="M22" s="16" t="inlineStr"/>
-      <c r="N22" s="16" t="inlineStr"/>
+      <c r="G22" s="17" t="inlineStr"/>
+      <c r="H22" s="17" t="inlineStr"/>
+      <c r="I22" s="17" t="inlineStr"/>
+      <c r="J22" s="17" t="inlineStr"/>
+      <c r="K22" s="17" t="inlineStr"/>
+      <c r="L22" s="17" t="inlineStr"/>
+      <c r="M22" s="17" t="inlineStr"/>
+      <c r="N22" s="17" t="inlineStr"/>
       <c r="O22" s="25" t="inlineStr">
         <is>
           <t>≈8.6人月</t>
@@ -1756,42 +1778,42 @@
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="20" t="inlineStr">
+      <c r="A23" s="21" t="inlineStr">
         <is>
           <t>ティー・エー・エス</t>
         </is>
       </c>
-      <c r="B23" s="21" t="inlineStr">
+      <c r="B23" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C23" s="21" t="inlineStr">
+      <c r="C23" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D23" s="21" t="n">
+      <c r="D23" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="E23" s="14" t="inlineStr">
+      <c r="E23" s="15" t="inlineStr">
         <is>
           <t>未割当</t>
         </is>
       </c>
-      <c r="F23" s="22" t="inlineStr">
+      <c r="F23" s="23" t="inlineStr">
         <is>
           <t>来期</t>
         </is>
       </c>
-      <c r="G23" s="16" t="inlineStr"/>
-      <c r="H23" s="16" t="inlineStr"/>
-      <c r="I23" s="16" t="inlineStr"/>
-      <c r="J23" s="16" t="inlineStr"/>
-      <c r="K23" s="16" t="inlineStr"/>
-      <c r="L23" s="16" t="inlineStr"/>
-      <c r="M23" s="16" t="inlineStr"/>
-      <c r="N23" s="16" t="inlineStr"/>
+      <c r="G23" s="17" t="inlineStr"/>
+      <c r="H23" s="17" t="inlineStr"/>
+      <c r="I23" s="17" t="inlineStr"/>
+      <c r="J23" s="17" t="inlineStr"/>
+      <c r="K23" s="17" t="inlineStr"/>
+      <c r="L23" s="17" t="inlineStr"/>
+      <c r="M23" s="17" t="inlineStr"/>
+      <c r="N23" s="17" t="inlineStr"/>
       <c r="O23" s="25" t="inlineStr">
         <is>
           <t>≈5人月</t>
@@ -1854,7 +1876,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C24" s="13" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1862,24 +1884,24 @@
       <c r="D24" s="13" t="n">
         <v>2.35</v>
       </c>
-      <c r="E24" s="14" t="inlineStr">
+      <c r="E24" s="15" t="inlineStr">
         <is>
           <t>未割当</t>
         </is>
       </c>
-      <c r="F24" s="23" t="inlineStr">
-        <is>
-          <t>来期・小さめ</t>
-        </is>
-      </c>
-      <c r="G24" s="16" t="inlineStr"/>
-      <c r="H24" s="16" t="inlineStr"/>
-      <c r="I24" s="16" t="inlineStr"/>
-      <c r="J24" s="16" t="inlineStr"/>
-      <c r="K24" s="16" t="inlineStr"/>
-      <c r="L24" s="16" t="inlineStr"/>
-      <c r="M24" s="16" t="inlineStr"/>
-      <c r="N24" s="16" t="inlineStr"/>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>来期</t>
+        </is>
+      </c>
+      <c r="G24" s="17" t="inlineStr"/>
+      <c r="H24" s="17" t="inlineStr"/>
+      <c r="I24" s="17" t="inlineStr"/>
+      <c r="J24" s="17" t="inlineStr"/>
+      <c r="K24" s="17" t="inlineStr"/>
+      <c r="L24" s="17" t="inlineStr"/>
+      <c r="M24" s="17" t="inlineStr"/>
+      <c r="N24" s="17" t="inlineStr"/>
       <c r="O24" s="25" t="inlineStr">
         <is>
           <t>≈2.35</t>
@@ -1932,32 +1954,32 @@
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="20" t="inlineStr">
+      <c r="A25" s="21" t="inlineStr">
         <is>
           <t>アーク</t>
         </is>
       </c>
-      <c r="B25" s="21" t="inlineStr">
+      <c r="B25" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C25" s="21" t="inlineStr">
+      <c r="C25" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D25" s="21" t="n">
+      <c r="D25" s="22" t="n">
         <v>0.7</v>
       </c>
-      <c r="E25" s="14" t="inlineStr">
+      <c r="E25" s="15" t="inlineStr">
         <is>
           <t>未割当</t>
         </is>
       </c>
-      <c r="F25" s="22" t="inlineStr">
-        <is>
-          <t>未定・隙間</t>
+      <c r="F25" s="23" t="inlineStr">
+        <is>
+          <t>来期</t>
         </is>
       </c>
       <c r="G25" s="25" t="inlineStr">
@@ -2052,68 +2074,68 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="26" t="inlineStr">
+      <c r="A26" s="27" t="inlineStr">
         <is>
           <t>合計（概算）</t>
         </is>
       </c>
-      <c r="B26" s="27" t="inlineStr">
+      <c r="B26" s="28" t="inlineStr">
         <is>
           <t>≈20</t>
         </is>
       </c>
-      <c r="C26" s="28" t="inlineStr">
+      <c r="C26" s="29" t="inlineStr">
         <is>
           <t>RD人月</t>
         </is>
       </c>
-      <c r="D26" s="29" t="inlineStr">
-        <is>
-          <t>≈112</t>
-        </is>
-      </c>
-      <c r="E26" s="30" t="inlineStr">
-        <is>
-          <t>Dev人月（東洋捺染40含む）※灰帯の数字が未定時期の工数</t>
-        </is>
-      </c>
-      <c r="G26" s="31" t="n"/>
-      <c r="H26" s="31" t="n"/>
-      <c r="I26" s="31" t="n"/>
-      <c r="J26" s="31" t="n"/>
-      <c r="K26" s="31" t="n"/>
-      <c r="L26" s="31" t="n"/>
-      <c r="M26" s="31" t="n"/>
-      <c r="N26" s="31" t="n"/>
-      <c r="O26" s="31" t="n"/>
-      <c r="P26" s="31" t="n"/>
-      <c r="Q26" s="31" t="n"/>
-      <c r="R26" s="31" t="n"/>
-      <c r="S26" s="31" t="n"/>
-      <c r="T26" s="31" t="n"/>
-      <c r="U26" s="31" t="n"/>
-      <c r="V26" s="31" t="n"/>
-      <c r="W26" s="31" t="n"/>
-      <c r="X26" s="31" t="n"/>
+      <c r="D26" s="30" t="inlineStr">
+        <is>
+          <t>≈111.35</t>
+        </is>
+      </c>
+      <c r="E26" s="31" t="inlineStr">
+        <is>
+          <t>Dev人月（豊商事4反映／東洋捺染40含む）※灰帯=時期未定の工数</t>
+        </is>
+      </c>
+      <c r="G26" s="32" t="n"/>
+      <c r="H26" s="32" t="n"/>
+      <c r="I26" s="32" t="n"/>
+      <c r="J26" s="32" t="n"/>
+      <c r="K26" s="32" t="n"/>
+      <c r="L26" s="32" t="n"/>
+      <c r="M26" s="32" t="n"/>
+      <c r="N26" s="32" t="n"/>
+      <c r="O26" s="32" t="n"/>
+      <c r="P26" s="32" t="n"/>
+      <c r="Q26" s="32" t="n"/>
+      <c r="R26" s="32" t="n"/>
+      <c r="S26" s="32" t="n"/>
+      <c r="T26" s="32" t="n"/>
+      <c r="U26" s="32" t="n"/>
+      <c r="V26" s="32" t="n"/>
+      <c r="W26" s="32" t="n"/>
+      <c r="X26" s="32" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>③ 川手・小園の月次負荷（キャパ2.0人月/月）</t>
+          <t>③ 担当者別・月次負荷（1人キャパ=1.0人月/月／工数は担当人数で按分）</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>神鋼・アムリードは時期未定のため未算入（灰帯の隠し負荷に注意）</t>
+          <t>神鋼・アムリードは時期未定のため未算入。東洋捺染を川手・佐久間にした結果、小園の10〜12月は改善、川手はなお超過。</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="inlineStr">
-        <is>
-          <t>指標</t>
+      <c r="A30" s="33" t="inlineStr">
+        <is>
+          <t>担当</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
@@ -2156,151 +2178,160 @@
           <t>27/3</t>
         </is>
       </c>
+      <c r="J30" s="33" t="inlineStr">
+        <is>
+          <t>判定</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="26" t="inlineStr">
-        <is>
-          <t>負荷</t>
-        </is>
-      </c>
-      <c r="B31" s="32" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="C31" s="32" t="n">
-        <v>1.5</v>
+      <c r="A31" s="34" t="inlineStr">
+        <is>
+          <t>川手</t>
+        </is>
+      </c>
+      <c r="B31" s="35" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="C31" s="35" t="n">
+        <v>0.75</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>3.7</v>
+        <v>1.84</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="F31" s="33" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="G31" s="34" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="G31" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="34" t="n">
+      <c r="H31" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="I31" s="34" t="n">
+      <c r="I31" s="13" t="n">
         <v>0</v>
       </c>
+      <c r="J31" s="16" t="inlineStr">
+        <is>
+          <t>10〜12月超過</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="26" t="inlineStr">
-        <is>
-          <t>キャパ</t>
+      <c r="A32" s="36" t="inlineStr">
+        <is>
+          <t>小園</t>
         </is>
       </c>
       <c r="B32" s="35" t="n">
-        <v>2</v>
+        <v>0.75</v>
       </c>
       <c r="C32" s="35" t="n">
-        <v>2</v>
-      </c>
-      <c r="D32" s="35" t="n">
-        <v>2</v>
-      </c>
-      <c r="E32" s="35" t="n">
-        <v>2</v>
+        <v>0.75</v>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>1.17</v>
       </c>
       <c r="F32" s="35" t="n">
-        <v>2</v>
-      </c>
-      <c r="G32" s="35" t="n">
-        <v>2</v>
-      </c>
-      <c r="H32" s="35" t="n">
-        <v>2</v>
-      </c>
-      <c r="I32" s="35" t="n">
-        <v>2</v>
+        <v>0.67</v>
+      </c>
+      <c r="G32" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="16" t="inlineStr">
+        <is>
+          <t>10〜11月やや超過</t>
+        </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="26" t="inlineStr">
-        <is>
-          <t>過不足</t>
-        </is>
-      </c>
-      <c r="B33" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C33" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D33" s="4" t="n">
-        <v>-1.7</v>
-      </c>
-      <c r="E33" s="4" t="n">
-        <v>-1.7</v>
-      </c>
-      <c r="F33" s="4" t="n">
-        <v>-0.7</v>
-      </c>
-      <c r="G33" s="32" t="n">
-        <v>2</v>
-      </c>
-      <c r="H33" s="32" t="n">
-        <v>2</v>
-      </c>
-      <c r="I33" s="32" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="34" ht="32" customHeight="1">
-      <c r="A34" s="26" t="inlineStr">
-        <is>
-          <t>中身</t>
-        </is>
-      </c>
-      <c r="B34" s="36" t="inlineStr">
-        <is>
-          <t>ローリングスRD</t>
-        </is>
-      </c>
-      <c r="C34" s="36" t="inlineStr">
-        <is>
-          <t>ローリングスRD</t>
-        </is>
-      </c>
-      <c r="D34" s="36" t="inlineStr">
-        <is>
-          <t>イシダ+三菱+東洋</t>
-        </is>
-      </c>
-      <c r="E34" s="36" t="inlineStr">
-        <is>
-          <t>イシダ+三菱+東洋</t>
-        </is>
-      </c>
-      <c r="F34" s="36" t="inlineStr">
-        <is>
-          <t>三菱+東洋</t>
-        </is>
-      </c>
-      <c r="G34" s="36" t="inlineStr">
-        <is>
-          <t>Dev未割当</t>
-        </is>
-      </c>
-      <c r="H34" s="36" t="inlineStr">
-        <is>
-          <t>Dev未割当</t>
-        </is>
-      </c>
-      <c r="I34" s="36" t="inlineStr">
-        <is>
-          <t>Dev未割当</t>
+      <c r="A33" s="37" t="inlineStr">
+        <is>
+          <t>佐久間</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="35" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="E33" s="35" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="F33" s="35" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G33" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="23" t="inlineStr">
+        <is>
+          <t>東洋RDのみ・余裕あり</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="38" t="inlineStr">
+        <is>
+          <t>木村/森崎/伊藤</t>
+        </is>
+      </c>
+      <c r="B34" s="35" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C34" s="35" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D34" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="23" t="inlineStr">
+        <is>
+          <t>イワタニDev 1.5人月／成立</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="37" t="inlineStr">
-        <is>
-          <t>10〜12月 内訳</t>
+      <c r="A36" s="39" t="inlineStr">
+        <is>
+          <t>10〜12月 内訳（担当者別按分後）</t>
         </is>
       </c>
     </row>
@@ -2312,383 +2343,442 @@
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>期間</t>
+          <t>RD工数</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>RD</t>
+          <t>担当</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>月あたり</t>
+          <t>月あたり/人</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr">
         <is>
-          <t>10月</t>
+          <t>川手</t>
         </is>
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
-          <t>11月</t>
+          <t>小園</t>
         </is>
       </c>
       <c r="G37" s="10" t="inlineStr">
         <is>
-          <t>12月</t>
+          <t>佐久間</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="21" t="inlineStr">
-        <is>
-          <t>イシダ</t>
-        </is>
-      </c>
-      <c r="B38" s="21" t="inlineStr">
-        <is>
-          <t>10〜11</t>
-        </is>
-      </c>
-      <c r="C38" s="21" t="n">
+      <c r="A38" s="22" t="inlineStr">
+        <is>
+          <t>イシダ(10-11)</t>
+        </is>
+      </c>
+      <c r="B38" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="D38" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="F38" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="G38" s="21" t="n">
+      <c r="C38" s="22" t="inlineStr">
+        <is>
+          <t>川手・小園</t>
+        </is>
+      </c>
+      <c r="D38" s="22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E38" s="22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F38" s="22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G38" s="22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="21" t="inlineStr">
-        <is>
-          <t>三菱重工コンプレッサ</t>
-        </is>
-      </c>
-      <c r="B39" s="21" t="inlineStr">
-        <is>
-          <t>10〜12</t>
-        </is>
-      </c>
-      <c r="C39" s="21" t="n">
+      <c r="A39" s="22" t="inlineStr">
+        <is>
+          <t>三菱(10-12)</t>
+        </is>
+      </c>
+      <c r="B39" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="D39" s="21" t="n">
+      <c r="C39" s="22" t="inlineStr">
+        <is>
+          <t>川手・小園</t>
+        </is>
+      </c>
+      <c r="D39" s="22" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="E39" s="22" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="F39" s="22" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G39" s="22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="22" t="inlineStr">
+        <is>
+          <t>東洋捺染(10-12)</t>
+        </is>
+      </c>
+      <c r="B40" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C40" s="22" t="inlineStr">
+        <is>
+          <t>川手・佐久間</t>
+        </is>
+      </c>
+      <c r="D40" s="22" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="E40" s="22" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="F40" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="22" t="n">
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="40" t="inlineStr">
+        <is>
+          <t>合計 10〜11月</t>
+        </is>
+      </c>
+      <c r="B41" s="40" t="inlineStr"/>
+      <c r="C41" s="40" t="inlineStr"/>
+      <c r="D41" s="40" t="inlineStr"/>
+      <c r="E41" s="4" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="G41" s="41" t="n">
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="40" t="inlineStr">
+        <is>
+          <t>合計 12月</t>
+        </is>
+      </c>
+      <c r="B42" s="40" t="inlineStr"/>
+      <c r="C42" s="40" t="inlineStr"/>
+      <c r="D42" s="40" t="inlineStr"/>
+      <c r="E42" s="4" t="n">
         <v>1.33</v>
       </c>
-      <c r="E39" s="21" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="F39" s="21" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="G39" s="21" t="n">
-        <v>1.33</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="21" t="inlineStr">
-        <is>
-          <t>東洋捺染</t>
-        </is>
-      </c>
-      <c r="B40" s="21" t="inlineStr">
-        <is>
-          <t>10〜12</t>
-        </is>
-      </c>
-      <c r="C40" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="D40" s="21" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="E40" s="21" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="F40" s="21" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="G40" s="21" t="n">
-        <v>1.33</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="38" t="inlineStr">
-        <is>
-          <t>合計</t>
-        </is>
-      </c>
-      <c r="B41" s="38" t="inlineStr"/>
-      <c r="C41" s="38" t="n">
-        <v>10</v>
-      </c>
-      <c r="D41" s="38" t="inlineStr"/>
-      <c r="E41" s="4" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="F41" s="4" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="G41" s="4" t="n">
-        <v>2.7</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>④ 推奨アサイン・打ち手</t>
-        </is>
+      <c r="F42" s="41" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G42" s="41" t="n">
+        <v>0.67</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="39" t="inlineStr">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>④ 推奨アサイン・打ち手（見直し後）</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="33" t="inlineStr">
         <is>
           <t>時期</t>
         </is>
       </c>
-      <c r="B44" s="39" t="inlineStr">
-        <is>
-          <t>川手・小園</t>
-        </is>
-      </c>
-      <c r="C44" s="39" t="inlineStr">
-        <is>
-          <t>木村・森崎 or 他</t>
-        </is>
-      </c>
-      <c r="D44" s="39" t="inlineStr">
+      <c r="B45" s="33" t="inlineStr">
+        <is>
+          <t>川手</t>
+        </is>
+      </c>
+      <c r="C45" s="33" t="inlineStr">
+        <is>
+          <t>小園</t>
+        </is>
+      </c>
+      <c r="D45" s="33" t="inlineStr">
+        <is>
+          <t>佐久間 / 他</t>
+        </is>
+      </c>
+      <c r="E45" s="33" t="inlineStr">
         <is>
           <t>備考</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="22" t="inlineStr">
+    <row r="46" ht="28" customHeight="1">
+      <c r="A46" s="23" t="inlineStr">
         <is>
           <t>26/8〜9</t>
         </is>
       </c>
-      <c r="B45" s="22" t="inlineStr">
+      <c r="B46" s="23" t="inlineStr">
         <is>
           <t>ローリングス RD</t>
         </is>
       </c>
-      <c r="C45" s="22" t="inlineStr">
-        <is>
-          <t>イワタニ Dev</t>
-        </is>
-      </c>
-      <c r="D45" s="22" t="inlineStr">
-        <is>
-          <t>現状どおり成立</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="C46" s="23" t="inlineStr">
+        <is>
+          <t>ローリングス RD</t>
+        </is>
+      </c>
+      <c r="D46" s="23" t="inlineStr">
+        <is>
+          <t>イワタニ Dev（木村・森崎・伊藤）</t>
+        </is>
+      </c>
+      <c r="E46" s="23" t="inlineStr">
+        <is>
+          <t>成立</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="28" customHeight="1">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>26/10〜12</t>
         </is>
       </c>
-      <c r="B46" s="5" t="inlineStr">
-        <is>
-          <t>優先2案件のみ（例: イシダ＋東洋捺染）</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>ローリングスDev・豊商事</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>三菱RDはスライド候補 ←要決断</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="22" t="inlineStr">
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>イシダ+東洋（三菱は外す）</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>イシダ（+三菱は要判断）</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>東洋捺染 RD</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>川手超過解消には三菱スライドが有効</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="28" customHeight="1">
+      <c r="A48" s="23" t="inlineStr">
         <is>
           <t>27/1〜3</t>
         </is>
       </c>
-      <c r="B47" s="22" t="inlineStr">
-        <is>
-          <t>空き or スライドしたRD</t>
-        </is>
-      </c>
-      <c r="C47" s="22" t="inlineStr">
-        <is>
-          <t>イシダ Dev 4.5</t>
-        </is>
-      </c>
-      <c r="D47" s="22" t="inlineStr">
-        <is>
-          <t>開発担当を明示</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="22" t="inlineStr">
+      <c r="B48" s="23" t="inlineStr">
+        <is>
+          <t>スライドRDの受け皿</t>
+        </is>
+      </c>
+      <c r="C48" s="23" t="inlineStr">
+        <is>
+          <t>空き / 分析並行</t>
+        </is>
+      </c>
+      <c r="D48" s="23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E48" s="23" t="inlineStr">
+        <is>
+          <t>イシダDev4.5の担当を明示</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="28" customHeight="1">
+      <c r="A49" s="23" t="inlineStr">
         <is>
           <t>来期</t>
         </is>
       </c>
-      <c r="B48" s="22" t="inlineStr">
+      <c r="B49" s="23" t="inlineStr">
         <is>
           <t>高圧ガス等RDを四半期割</t>
         </is>
       </c>
-      <c r="C48" s="22" t="inlineStr">
-        <is>
-          <t>大型Devを複数名で消化</t>
-        </is>
-      </c>
-      <c r="D48" s="22" t="inlineStr">
-        <is>
-          <t>東洋捺染≈40は専用チーム化</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="37" t="inlineStr">
+      <c r="C49" s="23" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+      <c r="D49" s="23" t="inlineStr">
+        <is>
+          <t>東洋Dev専用チーム候補</t>
+        </is>
+      </c>
+      <c r="E49" s="23" t="inlineStr">
+        <is>
+          <t>Dev≈111のスロット化</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="39" t="inlineStr">
         <is>
           <t>打ち手チェック</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="40" t="inlineStr">
-        <is>
-          <t>□ 10〜12月のRDを最大2案件に制限する</t>
-        </is>
-      </c>
-    </row>
     <row r="52">
-      <c r="A52" s="40" t="inlineStr">
-        <is>
-          <t>□ ローリングスDev・豊商事の担当を川手・小園以外で決める</t>
+      <c r="A52" s="42" t="inlineStr">
+        <is>
+          <t>□ 三菱RDをスライドし、川手の10〜12月を1.0以下に落とす（最優先）</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="40" t="inlineStr">
-        <is>
-          <t>□ 東洋捺染≈40人月のフェーズ分割／専用チームを検討する</t>
+      <c r="A53" s="42" t="inlineStr">
+        <is>
+          <t>□ ローリングスDev 4.4・豊商事Dev 4・イシダDev 4.5 の担当を決める（未割当）</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="40" t="inlineStr">
-        <is>
-          <t>□ 来期案件（高圧ガス・日東・TG・三菱Dev・TAS等）を四半期スロット化する</t>
+      <c r="A54" s="42" t="inlineStr">
+        <is>
+          <t>□ 東洋捺染Dev≈40のフェーズ分割／専用チーム（佐久間起点）を検討</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="40" t="inlineStr">
-        <is>
-          <t>□ 神鋼商事・アムリードの時期を確定する（灰帯の隠し負荷）</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="37" t="inlineStr">
-        <is>
-          <t>担当者メモ</t>
+      <c r="A55" s="42" t="inlineStr">
+        <is>
+          <t>□ 来期案件を四半期スロット化（高圧ガス・日東・TG・三菱Dev・TAS等）</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="42" t="inlineStr">
+        <is>
+          <t>□ 神鋼商事・アムリードの時期を確定（川手・小園の隠し負荷）</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="39" t="inlineStr">
         <is>
+          <t>担当者メモ（見直し後）</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="33" t="inlineStr">
+        <is>
           <t>担当</t>
         </is>
       </c>
-      <c r="B58" s="39" t="inlineStr">
+      <c r="B59" s="33" t="inlineStr">
         <is>
           <t>今期の仕事</t>
         </is>
       </c>
-      <c r="C58" s="39" t="inlineStr">
-        <is>
-          <t>リスク</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="41" t="inlineStr">
+      <c r="C59" s="33" t="inlineStr">
+        <is>
+          <t>リスク / コメント</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="43" t="inlineStr">
         <is>
           <t>川手</t>
         </is>
       </c>
-      <c r="B59" s="22" t="inlineStr">
+      <c r="B60" s="23" t="inlineStr">
         <is>
           <t>ローリングスRD→イシダ/三菱/東洋RD（神鋼RDの可能性）</t>
         </is>
       </c>
-      <c r="C59" s="22" t="inlineStr">
-        <is>
-          <t>10〜12月が破綻しやすい</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="41" t="inlineStr">
+      <c r="C60" s="23" t="inlineStr">
+        <is>
+          <t>10〜12月が最大ボトルネック。三菱外しが効く</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="44" t="inlineStr">
         <is>
           <t>小園</t>
         </is>
       </c>
-      <c r="B60" s="22" t="inlineStr">
-        <is>
-          <t>同上（神鋼は川手のみ記載）</t>
-        </is>
-      </c>
-      <c r="C60" s="22" t="inlineStr">
-        <is>
-          <t>同上</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="22" t="inlineStr">
-        <is>
-          <t>木村・森崎</t>
-        </is>
-      </c>
-      <c r="B61" s="22" t="inlineStr">
-        <is>
-          <t>イワタニ8〜9月のみ</t>
-        </is>
-      </c>
-      <c r="C61" s="22" t="inlineStr">
-        <is>
-          <t>今期後半〜来期の開発プール候補</t>
+      <c r="B61" s="23" t="inlineStr">
+        <is>
+          <t>ローリングスRD→イシダ/三菱RD（東洋からは外れ）</t>
+        </is>
+      </c>
+      <c r="C61" s="23" t="inlineStr">
+        <is>
+          <t>以前より改善。イシダ+三菱で10〜11月はなお逼迫</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="42" t="inlineStr">
+      <c r="A62" s="45" t="inlineStr">
+        <is>
+          <t>佐久間</t>
+        </is>
+      </c>
+      <c r="B62" s="23" t="inlineStr">
+        <is>
+          <t>東洋捺染RD（10〜12）</t>
+        </is>
+      </c>
+      <c r="C62" s="23" t="inlineStr">
+        <is>
+          <t>新規投入。余裕あり。東洋Devの受け皿候補</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="23" t="inlineStr">
+        <is>
+          <t>木村・森崎・伊藤</t>
+        </is>
+      </c>
+      <c r="B63" s="23" t="inlineStr">
+        <is>
+          <t>イワタニDev 8〜9月</t>
+        </is>
+      </c>
+      <c r="C63" s="23" t="inlineStr">
+        <is>
+          <t>成立。後半の未割当Devプール候補</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="15" t="inlineStr">
         <is>
           <t>未割当</t>
         </is>
       </c>
-      <c r="B62" s="22" t="inlineStr">
-        <is>
-          <t>開発の大半≈112人月</t>
-        </is>
-      </c>
-      <c r="C62" s="22" t="inlineStr">
+      <c r="B64" s="23" t="inlineStr">
+        <is>
+          <t>Dev合計≈111.35人月</t>
+        </is>
+      </c>
+      <c r="C64" s="23" t="inlineStr">
         <is>
           <t>来期リソース計画が本丸</t>
         </is>
@@ -2697,22 +2787,22 @@
   </sheetData>
   <mergeCells count="17">
     <mergeCell ref="A2:V2"/>
+    <mergeCell ref="A56:H56"/>
+    <mergeCell ref="B5:N5"/>
     <mergeCell ref="A10:V10"/>
     <mergeCell ref="A28:V28"/>
-    <mergeCell ref="A29:L29"/>
     <mergeCell ref="A53:H53"/>
-    <mergeCell ref="B6:L6"/>
     <mergeCell ref="A55:H55"/>
+    <mergeCell ref="A44:V44"/>
     <mergeCell ref="A1:V1"/>
-    <mergeCell ref="B7:L7"/>
-    <mergeCell ref="A51:H51"/>
+    <mergeCell ref="A54:H54"/>
     <mergeCell ref="A52:H52"/>
-    <mergeCell ref="A54:H54"/>
-    <mergeCell ref="B5:L5"/>
+    <mergeCell ref="A29:N29"/>
     <mergeCell ref="A9:V9"/>
     <mergeCell ref="E26:F26"/>
+    <mergeCell ref="B7:N7"/>
+    <mergeCell ref="B6:N6"/>
     <mergeCell ref="A4:V4"/>
-    <mergeCell ref="A43:V43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Simplify gantt legend to R/D with monthly headcount
- Remove U; Dev assignee column white=assigned, yellow=unassigned
- Each month cell shows people needed (MM / months)
- Add monthly headcount total row

Co-authored-by: kozonoflight <kozonoflight@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/knowledge/人積み/2026-2027_案件人積み.xlsx
+++ b/knowledge/人積み/2026-2027_案件人積み.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -78,12 +78,13 @@
       <name val="Yu Gothic"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="8"/>
+      <sz val="7"/>
     </font>
     <font>
       <name val="Yu Gothic"/>
       <b val="1"/>
-      <sz val="8"/>
+      <color rgb="001A1A1A"/>
+      <sz val="7"/>
     </font>
     <font>
       <name val="Yu Gothic"/>
@@ -91,8 +92,13 @@
       <color rgb="00333333"/>
       <sz val="7"/>
     </font>
+    <font>
+      <name val="Yu Gothic"/>
+      <b val="1"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="19">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -151,12 +157,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="0070AD47"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFFBF0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0070AD47"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -211,7 +222,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -249,7 +260,7 @@
     <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -261,10 +272,10 @@
     <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -276,52 +287,61 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="16" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -689,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X64"/>
+  <dimension ref="A1:X69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -718,24 +738,24 @@
     <col width="5.8" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>案件人積み・スケジュール俯瞰（1シート完結）※割当見直し反映</t>
+          <t>案件人積み・スケジュール俯瞰（1シート完結）</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>更新: 豊商事Dev=4人月 / 東洋捺染RD=川手・佐久間 / イワタニDev=木村・森崎（伊藤）。負荷は担当者別に再計算（工数は担当人数で按分）。</t>
+          <t>ガント数字=その月に必要な人数（人月÷月数）。R=要件定義 / D=開発。Dev担当が白=割当済・黄=未割当。灰帯=時期未定。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>① 一目サマリ（見直し後）</t>
+          <t>① 一目サマリ</t>
         </is>
       </c>
     </row>
@@ -747,7 +767,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>26/10〜12：川手が3案件同時（イシダ・三菱・東洋捺染）で月≈1.8人月超。小園は東洋から外れ≈1.2まで改善も、イシダ+三菱でなお逼迫</t>
+          <t>26/10〜12：川手が3案件同時（イシダ・三菱・東洋）で月≈1.8人月超。小園は東洋外れで≈1.2まで改善も、イシダ+三菱でなお逼迫</t>
         </is>
       </c>
     </row>
@@ -759,7 +779,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>東洋捺染RDに佐久間を投入 → 小園の10〜12月負荷が軽減。豊商事Dev 6→4人月で未割当Dev合計≈111.35</t>
+          <t>東洋捺染RD=川手・佐久間。豊商事Dev=4人月。イワタニ=木村・森崎（伊藤）</t>
         </is>
       </c>
     </row>
@@ -771,21 +791,21 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>開発の大半が未割当。ローリングスDev・豊商事・イシダDevの担当決めが必要。神鋼・アムリードは時期未定の隠し負荷</t>
+          <t>Dev担当が黄色い案件は未割当。ローリングス/豊商事/イシダDev等の担当決めが必要</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>② 簡易ガント</t>
+          <t>② 簡易ガント（セル内の数字＝その月に必要な人数）</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>凡例: R=要件定義 / D=開発・担当あり / U=開発・未割当 / 灰+数字=時期未定だが工数判明 / 黄列ヘッダ=来期</t>
+          <t>凡例: R=要件定義(青) / D=開発(緑) / 灰=時期未定の開発or混合。数字は必要人数/月。Dev担当列: 白=割当完了 / 黄=未割当</t>
         </is>
       </c>
     </row>
@@ -911,7 +931,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1">
+    <row r="12" ht="28" customHeight="1">
       <c r="A12" s="12" t="inlineStr">
         <is>
           <t>イシダ</t>
@@ -942,28 +962,33 @@
       <c r="H12" s="17" t="inlineStr"/>
       <c r="I12" s="18" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>R
+1人</t>
         </is>
       </c>
       <c r="J12" s="18" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>R
+1人</t>
         </is>
       </c>
       <c r="K12" s="17" t="inlineStr"/>
       <c r="L12" s="19" t="inlineStr">
         <is>
-          <t>U4.5</t>
+          <t>D
+1.5人</t>
         </is>
       </c>
       <c r="M12" s="19" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>D
+1.5人</t>
         </is>
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>D
+1.5人</t>
         </is>
       </c>
       <c r="O12" s="20" t="inlineStr"/>
@@ -977,7 +1002,7 @@
       <c r="W12" s="20" t="inlineStr"/>
       <c r="X12" s="20" t="inlineStr"/>
     </row>
-    <row r="13" ht="22" customHeight="1">
+    <row r="13" ht="28" customHeight="1">
       <c r="A13" s="21" t="inlineStr">
         <is>
           <t>ローリングスジャパン</t>
@@ -1006,27 +1031,32 @@
       </c>
       <c r="G13" s="18" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>R
+1.5人</t>
         </is>
       </c>
       <c r="H13" s="18" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>R
+1.5人</t>
         </is>
       </c>
       <c r="I13" s="19" t="inlineStr">
         <is>
-          <t>U4.4</t>
+          <t>D
+1.5人</t>
         </is>
       </c>
       <c r="J13" s="19" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>D
+1.5人</t>
         </is>
       </c>
       <c r="K13" s="19" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>D
+1.5人</t>
         </is>
       </c>
       <c r="L13" s="17" t="inlineStr"/>
@@ -1043,7 +1073,7 @@
       <c r="W13" s="20" t="inlineStr"/>
       <c r="X13" s="20" t="inlineStr"/>
     </row>
-    <row r="14" ht="22" customHeight="1">
+    <row r="14" ht="28" customHeight="1">
       <c r="A14" s="12" t="inlineStr">
         <is>
           <t>イワタニ・ケンボロー</t>
@@ -1062,7 +1092,7 @@
       <c r="D14" s="13" t="n">
         <v>1.5</v>
       </c>
-      <c r="E14" s="14" t="inlineStr">
+      <c r="E14" s="24" t="inlineStr">
         <is>
           <t>木村・森崎（伊藤）</t>
         </is>
@@ -1072,14 +1102,16 @@
           <t>成立</t>
         </is>
       </c>
-      <c r="G14" s="24" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="H14" s="24" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="G14" s="19" t="inlineStr">
+        <is>
+          <t>D
+0.8人</t>
+        </is>
+      </c>
+      <c r="H14" s="19" t="inlineStr">
+        <is>
+          <t>D
+0.8人</t>
         </is>
       </c>
       <c r="I14" s="17" t="inlineStr"/>
@@ -1099,7 +1131,7 @@
       <c r="W14" s="20" t="inlineStr"/>
       <c r="X14" s="20" t="inlineStr"/>
     </row>
-    <row r="15" ht="22" customHeight="1">
+    <row r="15" ht="28" customHeight="1">
       <c r="A15" s="21" t="inlineStr">
         <is>
           <t>豊商事</t>
@@ -1131,22 +1163,26 @@
       <c r="G15" s="17" t="inlineStr"/>
       <c r="H15" s="19" t="inlineStr">
         <is>
-          <t>U≈4</t>
+          <t>D
+1人</t>
         </is>
       </c>
       <c r="I15" s="19" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>D
+1人</t>
         </is>
       </c>
       <c r="J15" s="19" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>D
+1人</t>
         </is>
       </c>
       <c r="K15" s="19" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>D
+1人</t>
         </is>
       </c>
       <c r="L15" s="17" t="inlineStr"/>
@@ -1163,7 +1199,7 @@
       <c r="W15" s="20" t="inlineStr"/>
       <c r="X15" s="20" t="inlineStr"/>
     </row>
-    <row r="16" ht="22" customHeight="1">
+    <row r="16" ht="28" customHeight="1">
       <c r="A16" s="12" t="inlineStr">
         <is>
           <t>三菱重工コンプレッサ</t>
@@ -1194,17 +1230,20 @@
       <c r="H16" s="17" t="inlineStr"/>
       <c r="I16" s="18" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>R
+1.3人</t>
         </is>
       </c>
       <c r="J16" s="18" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>R
+1.3人</t>
         </is>
       </c>
       <c r="K16" s="18" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>R
+1.3人</t>
         </is>
       </c>
       <c r="L16" s="17" t="inlineStr"/>
@@ -1212,56 +1251,66 @@
       <c r="N16" s="17" t="inlineStr"/>
       <c r="O16" s="25" t="inlineStr">
         <is>
-          <t>≈10人月</t>
+          <t>D
+1人</t>
         </is>
       </c>
       <c r="P16" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+1人</t>
         </is>
       </c>
       <c r="Q16" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+1人</t>
         </is>
       </c>
       <c r="R16" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+1人</t>
         </is>
       </c>
       <c r="S16" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+1人</t>
         </is>
       </c>
       <c r="T16" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+1人</t>
         </is>
       </c>
       <c r="U16" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+1人</t>
         </is>
       </c>
       <c r="V16" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+1人</t>
         </is>
       </c>
       <c r="W16" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+1人</t>
         </is>
       </c>
       <c r="X16" s="25" t="inlineStr">
         <is>
-          <t>…</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
+          <t>D
+1人</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
       <c r="A17" s="21" t="inlineStr">
         <is>
           <t>東洋捺染</t>
@@ -1292,17 +1341,20 @@
       <c r="H17" s="17" t="inlineStr"/>
       <c r="I17" s="18" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>R
+1.3人</t>
         </is>
       </c>
       <c r="J17" s="18" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>R
+1.3人</t>
         </is>
       </c>
       <c r="K17" s="18" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>R
+1.3人</t>
         </is>
       </c>
       <c r="L17" s="17" t="inlineStr"/>
@@ -1310,56 +1362,66 @@
       <c r="N17" s="17" t="inlineStr"/>
       <c r="O17" s="25" t="inlineStr">
         <is>
-          <t>≈40人月</t>
+          <t>D
+4人</t>
         </is>
       </c>
       <c r="P17" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+4人</t>
         </is>
       </c>
       <c r="Q17" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+4人</t>
         </is>
       </c>
       <c r="R17" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+4人</t>
         </is>
       </c>
       <c r="S17" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+4人</t>
         </is>
       </c>
       <c r="T17" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+4人</t>
         </is>
       </c>
       <c r="U17" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+4人</t>
         </is>
       </c>
       <c r="V17" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+4人</t>
         </is>
       </c>
       <c r="W17" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+4人</t>
         </is>
       </c>
       <c r="X17" s="25" t="inlineStr">
         <is>
-          <t>…</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
+          <t>D
+4人</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
       <c r="A18" s="12" t="inlineStr">
         <is>
           <t>神鋼商事</t>
@@ -1388,42 +1450,50 @@
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>RD1+Dev10</t>
+          <t>?
+1.4人</t>
         </is>
       </c>
       <c r="H18" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+1.4人</t>
         </is>
       </c>
       <c r="I18" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+1.4人</t>
         </is>
       </c>
       <c r="J18" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+1.4人</t>
         </is>
       </c>
       <c r="K18" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+1.4人</t>
         </is>
       </c>
       <c r="L18" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+1.4人</t>
         </is>
       </c>
       <c r="M18" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+1.4人</t>
         </is>
       </c>
       <c r="N18" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+1.4人</t>
         </is>
       </c>
       <c r="O18" s="20" t="inlineStr"/>
@@ -1437,7 +1507,7 @@
       <c r="W18" s="20" t="inlineStr"/>
       <c r="X18" s="20" t="inlineStr"/>
     </row>
-    <row r="19" ht="22" customHeight="1">
+    <row r="19" ht="28" customHeight="1">
       <c r="A19" s="21" t="inlineStr">
         <is>
           <t>アムリード</t>
@@ -1466,42 +1536,50 @@
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>RD3+Dev1.5</t>
+          <t>?
+0.6人</t>
         </is>
       </c>
       <c r="H19" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+0.6人</t>
         </is>
       </c>
       <c r="I19" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+0.6人</t>
         </is>
       </c>
       <c r="J19" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+0.6人</t>
         </is>
       </c>
       <c r="K19" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+0.6人</t>
         </is>
       </c>
       <c r="L19" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+0.6人</t>
         </is>
       </c>
       <c r="M19" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+0.6人</t>
         </is>
       </c>
       <c r="N19" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+0.6人</t>
         </is>
       </c>
       <c r="O19" s="20" t="inlineStr"/>
@@ -1515,7 +1593,7 @@
       <c r="W19" s="20" t="inlineStr"/>
       <c r="X19" s="20" t="inlineStr"/>
     </row>
-    <row r="20" ht="22" customHeight="1">
+    <row r="20" ht="28" customHeight="1">
       <c r="A20" s="12" t="inlineStr">
         <is>
           <t>高圧ガス工業</t>
@@ -1552,56 +1630,66 @@
       <c r="N20" s="17" t="inlineStr"/>
       <c r="O20" s="25" t="inlineStr">
         <is>
-          <t>RD3+Dev10</t>
+          <t>?
+1.3人</t>
         </is>
       </c>
       <c r="P20" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+1.3人</t>
         </is>
       </c>
       <c r="Q20" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+1.3人</t>
         </is>
       </c>
       <c r="R20" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+1.3人</t>
         </is>
       </c>
       <c r="S20" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+1.3人</t>
         </is>
       </c>
       <c r="T20" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+1.3人</t>
         </is>
       </c>
       <c r="U20" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+1.3人</t>
         </is>
       </c>
       <c r="V20" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+1.3人</t>
         </is>
       </c>
       <c r="W20" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>?
+1.3人</t>
         </is>
       </c>
       <c r="X20" s="25" t="inlineStr">
         <is>
-          <t>…</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
+          <t>?
+1.3人</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
       <c r="A21" s="21" t="inlineStr">
         <is>
           <t>日東電工BM</t>
@@ -1640,56 +1728,66 @@
       <c r="N21" s="17" t="inlineStr"/>
       <c r="O21" s="25" t="inlineStr">
         <is>
-          <t>≈8.8人月</t>
+          <t>D
+0.9人</t>
         </is>
       </c>
       <c r="P21" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.9人</t>
         </is>
       </c>
       <c r="Q21" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.9人</t>
         </is>
       </c>
       <c r="R21" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.9人</t>
         </is>
       </c>
       <c r="S21" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.9人</t>
         </is>
       </c>
       <c r="T21" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.9人</t>
         </is>
       </c>
       <c r="U21" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.9人</t>
         </is>
       </c>
       <c r="V21" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.9人</t>
         </is>
       </c>
       <c r="W21" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.9人</t>
         </is>
       </c>
       <c r="X21" s="25" t="inlineStr">
         <is>
-          <t>…</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
+          <t>D
+0.9人</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
       <c r="A22" s="12" t="inlineStr">
         <is>
           <t>TGソリューションズ</t>
@@ -1728,56 +1826,66 @@
       <c r="N22" s="17" t="inlineStr"/>
       <c r="O22" s="25" t="inlineStr">
         <is>
-          <t>≈8.6人月</t>
+          <t>D
+0.9人</t>
         </is>
       </c>
       <c r="P22" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.9人</t>
         </is>
       </c>
       <c r="Q22" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.9人</t>
         </is>
       </c>
       <c r="R22" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.9人</t>
         </is>
       </c>
       <c r="S22" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.9人</t>
         </is>
       </c>
       <c r="T22" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.9人</t>
         </is>
       </c>
       <c r="U22" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.9人</t>
         </is>
       </c>
       <c r="V22" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.9人</t>
         </is>
       </c>
       <c r="W22" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.9人</t>
         </is>
       </c>
       <c r="X22" s="25" t="inlineStr">
         <is>
-          <t>…</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
+          <t>D
+0.9人</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
       <c r="A23" s="21" t="inlineStr">
         <is>
           <t>ティー・エー・エス</t>
@@ -1816,56 +1924,66 @@
       <c r="N23" s="17" t="inlineStr"/>
       <c r="O23" s="25" t="inlineStr">
         <is>
-          <t>≈5人月</t>
+          <t>D
+0.5人</t>
         </is>
       </c>
       <c r="P23" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.5人</t>
         </is>
       </c>
       <c r="Q23" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.5人</t>
         </is>
       </c>
       <c r="R23" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.5人</t>
         </is>
       </c>
       <c r="S23" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.5人</t>
         </is>
       </c>
       <c r="T23" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.5人</t>
         </is>
       </c>
       <c r="U23" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.5人</t>
         </is>
       </c>
       <c r="V23" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.5人</t>
         </is>
       </c>
       <c r="W23" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.5人</t>
         </is>
       </c>
       <c r="X23" s="25" t="inlineStr">
         <is>
-          <t>…</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
+          <t>D
+0.5人</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
       <c r="A24" s="12" t="inlineStr">
         <is>
           <t>ニトムズ</t>
@@ -1904,56 +2022,66 @@
       <c r="N24" s="17" t="inlineStr"/>
       <c r="O24" s="25" t="inlineStr">
         <is>
-          <t>≈2.35</t>
+          <t>D
+0.2人</t>
         </is>
       </c>
       <c r="P24" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.2人</t>
         </is>
       </c>
       <c r="Q24" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.2人</t>
         </is>
       </c>
       <c r="R24" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.2人</t>
         </is>
       </c>
       <c r="S24" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.2人</t>
         </is>
       </c>
       <c r="T24" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.2人</t>
         </is>
       </c>
       <c r="U24" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.2人</t>
         </is>
       </c>
       <c r="V24" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.2人</t>
         </is>
       </c>
       <c r="W24" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.2人</t>
         </is>
       </c>
       <c r="X24" s="25" t="inlineStr">
         <is>
-          <t>…</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1">
+          <t>D
+0.2人</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="28" customHeight="1">
       <c r="A25" s="21" t="inlineStr">
         <is>
           <t>アーク</t>
@@ -1982,94 +2110,72 @@
           <t>来期</t>
         </is>
       </c>
-      <c r="G25" s="25" t="inlineStr">
-        <is>
-          <t>≈0.7人月</t>
-        </is>
-      </c>
-      <c r="H25" s="25" t="inlineStr">
-        <is>
-          <t>…</t>
-        </is>
-      </c>
-      <c r="I25" s="25" t="inlineStr">
-        <is>
-          <t>…</t>
-        </is>
-      </c>
-      <c r="J25" s="25" t="inlineStr">
-        <is>
-          <t>…</t>
-        </is>
-      </c>
-      <c r="K25" s="25" t="inlineStr">
-        <is>
-          <t>…</t>
-        </is>
-      </c>
-      <c r="L25" s="25" t="inlineStr">
-        <is>
-          <t>…</t>
-        </is>
-      </c>
-      <c r="M25" s="25" t="inlineStr">
-        <is>
-          <t>…</t>
-        </is>
-      </c>
-      <c r="N25" s="25" t="inlineStr">
-        <is>
-          <t>…</t>
-        </is>
-      </c>
+      <c r="G25" s="17" t="inlineStr"/>
+      <c r="H25" s="17" t="inlineStr"/>
+      <c r="I25" s="17" t="inlineStr"/>
+      <c r="J25" s="17" t="inlineStr"/>
+      <c r="K25" s="17" t="inlineStr"/>
+      <c r="L25" s="17" t="inlineStr"/>
+      <c r="M25" s="17" t="inlineStr"/>
+      <c r="N25" s="17" t="inlineStr"/>
       <c r="O25" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.1人</t>
         </is>
       </c>
       <c r="P25" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.1人</t>
         </is>
       </c>
       <c r="Q25" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.1人</t>
         </is>
       </c>
       <c r="R25" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.1人</t>
         </is>
       </c>
       <c r="S25" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.1人</t>
         </is>
       </c>
       <c r="T25" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.1人</t>
         </is>
       </c>
       <c r="U25" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.1人</t>
         </is>
       </c>
       <c r="V25" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.1人</t>
         </is>
       </c>
       <c r="W25" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.1人</t>
         </is>
       </c>
       <c r="X25" s="25" t="inlineStr">
         <is>
-          <t>…</t>
+          <t>D
+0.1人</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2202,7 @@
       </c>
       <c r="E26" s="31" t="inlineStr">
         <is>
-          <t>Dev人月（豊商事4反映／東洋捺染40含む）※灰帯=時期未定の工数</t>
+          <t>Dev人月合計。ガントの人数=工数÷月数。黄のDev担当=未割当</t>
         </is>
       </c>
       <c r="G26" s="32" t="n"/>
@@ -2128,7 +2234,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>神鋼・アムリードは時期未定のため未算入。東洋捺染を川手・佐久間にした結果、小園の10〜12月は改善、川手はなお超過。</t>
+          <t>神鋼・アムリードは時期未定のため未算入。東洋捺染を川手・佐久間にした結果、小園は改善、川手はなお超過。</t>
         </is>
       </c>
     </row>
@@ -2205,13 +2311,13 @@
       <c r="F31" s="4" t="n">
         <v>1.33</v>
       </c>
-      <c r="G31" s="13" t="n">
+      <c r="G31" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="13" t="n">
+      <c r="H31" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="I31" s="13" t="n">
+      <c r="I31" s="36" t="n">
         <v>0</v>
       </c>
       <c r="J31" s="16" t="inlineStr">
@@ -2221,7 +2327,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="36" t="inlineStr">
+      <c r="A32" s="37" t="inlineStr">
         <is>
           <t>小園</t>
         </is>
@@ -2241,13 +2347,13 @@
       <c r="F32" s="35" t="n">
         <v>0.67</v>
       </c>
-      <c r="G32" s="13" t="n">
+      <c r="G32" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="H32" s="13" t="n">
+      <c r="H32" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="I32" s="13" t="n">
+      <c r="I32" s="36" t="n">
         <v>0</v>
       </c>
       <c r="J32" s="16" t="inlineStr">
@@ -2257,15 +2363,15 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="37" t="inlineStr">
+      <c r="A33" s="38" t="inlineStr">
         <is>
           <t>佐久間</t>
         </is>
       </c>
-      <c r="B33" s="13" t="n">
+      <c r="B33" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="C33" s="13" t="n">
+      <c r="C33" s="36" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="35" t="n">
@@ -2277,13 +2383,13 @@
       <c r="F33" s="35" t="n">
         <v>0.67</v>
       </c>
-      <c r="G33" s="13" t="n">
+      <c r="G33" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="13" t="n">
+      <c r="H33" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="I33" s="13" t="n">
+      <c r="I33" s="36" t="n">
         <v>0</v>
       </c>
       <c r="J33" s="23" t="inlineStr">
@@ -2293,7 +2399,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="38" t="inlineStr">
+      <c r="A34" s="39" t="inlineStr">
         <is>
           <t>木村/森崎/伊藤</t>
         </is>
@@ -2304,32 +2410,32 @@
       <c r="C34" s="35" t="n">
         <v>0.25</v>
       </c>
-      <c r="D34" s="13" t="n">
+      <c r="D34" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="E34" s="13" t="n">
+      <c r="E34" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="F34" s="13" t="n">
+      <c r="F34" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="G34" s="13" t="n">
+      <c r="G34" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="13" t="n">
+      <c r="H34" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="I34" s="13" t="n">
+      <c r="I34" s="36" t="n">
         <v>0</v>
       </c>
       <c r="J34" s="23" t="inlineStr">
         <is>
-          <t>イワタニDev 1.5人月／成立</t>
+          <t>イワタニDev成立</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="39" t="inlineStr">
+      <c r="A36" s="40" t="inlineStr">
         <is>
           <t>10〜12月 内訳（担当者別按分後）</t>
         </is>
@@ -2353,7 +2459,7 @@
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>月あたり/人</t>
+          <t>必要人数/月</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr">
@@ -2386,8 +2492,10 @@
           <t>川手・小園</t>
         </is>
       </c>
-      <c r="D38" s="22" t="n">
-        <v>0.5</v>
+      <c r="D38" s="22" t="inlineStr">
+        <is>
+          <t>1.0人</t>
+        </is>
       </c>
       <c r="E38" s="22" t="n">
         <v>0.5</v>
@@ -2413,8 +2521,10 @@
           <t>川手・小園</t>
         </is>
       </c>
-      <c r="D39" s="22" t="n">
-        <v>0.67</v>
+      <c r="D39" s="22" t="inlineStr">
+        <is>
+          <t>1.3人</t>
+        </is>
       </c>
       <c r="E39" s="22" t="n">
         <v>0.67</v>
@@ -2440,8 +2550,10 @@
           <t>川手・佐久間</t>
         </is>
       </c>
-      <c r="D40" s="22" t="n">
-        <v>0.67</v>
+      <c r="D40" s="22" t="inlineStr">
+        <is>
+          <t>1.3人</t>
+        </is>
       </c>
       <c r="E40" s="22" t="n">
         <v>0.67</v>
@@ -2454,355 +2566,528 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="40" t="inlineStr">
-        <is>
-          <t>合計 10〜11月</t>
-        </is>
-      </c>
-      <c r="B41" s="40" t="inlineStr"/>
-      <c r="C41" s="40" t="inlineStr"/>
-      <c r="D41" s="40" t="inlineStr"/>
+      <c r="A41" s="41" t="inlineStr">
+        <is>
+          <t>合計 10〜11月(個人負荷)</t>
+        </is>
+      </c>
+      <c r="B41" s="41" t="inlineStr"/>
+      <c r="C41" s="41" t="inlineStr"/>
+      <c r="D41" s="41" t="inlineStr"/>
       <c r="E41" s="4" t="n">
         <v>1.84</v>
       </c>
       <c r="F41" s="4" t="n">
         <v>1.17</v>
       </c>
-      <c r="G41" s="41" t="n">
+      <c r="G41" s="35" t="n">
         <v>0.67</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="40" t="inlineStr">
-        <is>
-          <t>合計 12月</t>
-        </is>
-      </c>
-      <c r="B42" s="40" t="inlineStr"/>
-      <c r="C42" s="40" t="inlineStr"/>
-      <c r="D42" s="40" t="inlineStr"/>
+      <c r="A42" s="41" t="inlineStr">
+        <is>
+          <t>合計 12月(個人負荷)</t>
+        </is>
+      </c>
+      <c r="B42" s="41" t="inlineStr"/>
+      <c r="C42" s="41" t="inlineStr"/>
+      <c r="D42" s="41" t="inlineStr"/>
       <c r="E42" s="4" t="n">
         <v>1.33</v>
       </c>
-      <c r="F42" s="41" t="n">
+      <c r="F42" s="35" t="n">
         <v>0.67</v>
       </c>
-      <c r="G42" s="41" t="n">
+      <c r="G42" s="35" t="n">
         <v>0.67</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>④ 推奨アサイン・打ち手（見直し後）</t>
+      <c r="A44" s="40" t="inlineStr">
+        <is>
+          <t>月別・必要人数合計（全案件・時期が載っている帯のみ。灰の来期は参考）</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="33" t="inlineStr">
         <is>
+          <t>必要人数合計</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>26/8</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>26/9</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>26/10</t>
+        </is>
+      </c>
+      <c r="E45" s="10" t="inlineStr">
+        <is>
+          <t>26/11</t>
+        </is>
+      </c>
+      <c r="F45" s="10" t="inlineStr">
+        <is>
+          <t>26/12</t>
+        </is>
+      </c>
+      <c r="G45" s="10" t="inlineStr">
+        <is>
+          <t>27/1</t>
+        </is>
+      </c>
+      <c r="H45" s="10" t="inlineStr">
+        <is>
+          <t>27/2</t>
+        </is>
+      </c>
+      <c r="I45" s="10" t="inlineStr">
+        <is>
+          <t>27/3</t>
+        </is>
+      </c>
+      <c r="J45" s="42" t="inlineStr">
+        <is>
+          <t>27/4</t>
+        </is>
+      </c>
+      <c r="K45" s="42" t="inlineStr">
+        <is>
+          <t>27/5</t>
+        </is>
+      </c>
+      <c r="L45" s="42" t="inlineStr">
+        <is>
+          <t>27/6</t>
+        </is>
+      </c>
+      <c r="M45" s="42" t="inlineStr">
+        <is>
+          <t>27/7</t>
+        </is>
+      </c>
+      <c r="N45" s="42" t="inlineStr">
+        <is>
+          <t>27/8</t>
+        </is>
+      </c>
+      <c r="O45" s="42" t="inlineStr">
+        <is>
+          <t>27/9</t>
+        </is>
+      </c>
+      <c r="P45" s="42" t="inlineStr">
+        <is>
+          <t>27/10</t>
+        </is>
+      </c>
+      <c r="Q45" s="42" t="inlineStr">
+        <is>
+          <t>27/11</t>
+        </is>
+      </c>
+      <c r="R45" s="42" t="inlineStr">
+        <is>
+          <t>27/12</t>
+        </is>
+      </c>
+      <c r="S45" s="42" t="inlineStr">
+        <is>
+          <t>28/1</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="27" t="inlineStr">
+        <is>
+          <t>合計(人)</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="C46" s="4" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="D46" s="4" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="F46" s="4" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="G46" s="43" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H46" s="43" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I46" s="43" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J46" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="K46" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="L46" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="M46" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="N46" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="O46" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="P46" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q46" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="R46" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="S46" s="4" t="n">
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>※上段ガントの各セル人数を月ごとに合算。同じ月に複数案件が重なると必要な延べ人数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>④ 推奨アサイン・打ち手</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="33" t="inlineStr">
+        <is>
           <t>時期</t>
         </is>
       </c>
-      <c r="B45" s="33" t="inlineStr">
+      <c r="B50" s="33" t="inlineStr">
         <is>
           <t>川手</t>
         </is>
       </c>
-      <c r="C45" s="33" t="inlineStr">
+      <c r="C50" s="33" t="inlineStr">
         <is>
           <t>小園</t>
         </is>
       </c>
-      <c r="D45" s="33" t="inlineStr">
+      <c r="D50" s="33" t="inlineStr">
         <is>
           <t>佐久間 / 他</t>
         </is>
       </c>
-      <c r="E45" s="33" t="inlineStr">
+      <c r="E50" s="33" t="inlineStr">
         <is>
           <t>備考</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="28" customHeight="1">
-      <c r="A46" s="23" t="inlineStr">
+    <row r="51" ht="28" customHeight="1">
+      <c r="A51" s="23" t="inlineStr">
         <is>
           <t>26/8〜9</t>
         </is>
       </c>
-      <c r="B46" s="23" t="inlineStr">
+      <c r="B51" s="23" t="inlineStr">
         <is>
           <t>ローリングス RD</t>
         </is>
       </c>
-      <c r="C46" s="23" t="inlineStr">
+      <c r="C51" s="23" t="inlineStr">
         <is>
           <t>ローリングス RD</t>
         </is>
       </c>
-      <c r="D46" s="23" t="inlineStr">
+      <c r="D51" s="23" t="inlineStr">
         <is>
           <t>イワタニ Dev（木村・森崎・伊藤）</t>
         </is>
       </c>
-      <c r="E46" s="23" t="inlineStr">
+      <c r="E51" s="23" t="inlineStr">
         <is>
           <t>成立</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="28" customHeight="1">
-      <c r="A47" s="5" t="inlineStr">
+    <row r="52" ht="28" customHeight="1">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>26/10〜12</t>
         </is>
       </c>
-      <c r="B47" s="5" t="inlineStr">
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>イシダ+東洋（三菱は外す）</t>
         </is>
       </c>
-      <c r="C47" s="5" t="inlineStr">
+      <c r="C52" s="5" t="inlineStr">
         <is>
           <t>イシダ（+三菱は要判断）</t>
         </is>
       </c>
-      <c r="D47" s="5" t="inlineStr">
+      <c r="D52" s="5" t="inlineStr">
         <is>
           <t>東洋捺染 RD</t>
         </is>
       </c>
-      <c r="E47" s="5" t="inlineStr">
+      <c r="E52" s="5" t="inlineStr">
         <is>
           <t>川手超過解消には三菱スライドが有効</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="28" customHeight="1">
-      <c r="A48" s="23" t="inlineStr">
+    <row r="53" ht="28" customHeight="1">
+      <c r="A53" s="23" t="inlineStr">
         <is>
           <t>27/1〜3</t>
         </is>
       </c>
-      <c r="B48" s="23" t="inlineStr">
+      <c r="B53" s="23" t="inlineStr">
         <is>
           <t>スライドRDの受け皿</t>
         </is>
       </c>
-      <c r="C48" s="23" t="inlineStr">
+      <c r="C53" s="23" t="inlineStr">
         <is>
           <t>空き / 分析並行</t>
         </is>
       </c>
-      <c r="D48" s="23" t="inlineStr">
+      <c r="D53" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E48" s="23" t="inlineStr">
-        <is>
-          <t>イシダDev4.5の担当を明示</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="28" customHeight="1">
-      <c r="A49" s="23" t="inlineStr">
+      <c r="E53" s="23" t="inlineStr">
+        <is>
+          <t>イシダDevの担当を明示（Dev担当を白に）</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="28" customHeight="1">
+      <c r="A54" s="23" t="inlineStr">
         <is>
           <t>来期</t>
         </is>
       </c>
-      <c r="B49" s="23" t="inlineStr">
+      <c r="B54" s="23" t="inlineStr">
         <is>
           <t>高圧ガス等RDを四半期割</t>
         </is>
       </c>
-      <c r="C49" s="23" t="inlineStr">
+      <c r="C54" s="23" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
-      <c r="D49" s="23" t="inlineStr">
+      <c r="D54" s="23" t="inlineStr">
         <is>
           <t>東洋Dev専用チーム候補</t>
         </is>
       </c>
-      <c r="E49" s="23" t="inlineStr">
-        <is>
-          <t>Dev≈111のスロット化</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="39" t="inlineStr">
+      <c r="E54" s="23" t="inlineStr">
+        <is>
+          <t>黄のDev担当を潰していく</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="40" t="inlineStr">
         <is>
           <t>打ち手チェック</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="42" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="44" t="inlineStr">
         <is>
           <t>□ 三菱RDをスライドし、川手の10〜12月を1.0以下に落とす（最優先）</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="42" t="inlineStr">
-        <is>
-          <t>□ ローリングスDev 4.4・豊商事Dev 4・イシダDev 4.5 の担当を決める（未割当）</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="42" t="inlineStr">
-        <is>
-          <t>□ 東洋捺染Dev≈40のフェーズ分割／専用チーム（佐久間起点）を検討</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="42" t="inlineStr">
-        <is>
-          <t>□ 来期案件を四半期スロット化（高圧ガス・日東・TG・三菱Dev・TAS等）</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="42" t="inlineStr">
-        <is>
-          <t>□ 神鋼商事・アムリードの時期を確定（川手・小園の隠し負荷）</t>
-        </is>
-      </c>
-    </row>
     <row r="58">
-      <c r="A58" s="39" t="inlineStr">
-        <is>
-          <t>担当者メモ（見直し後）</t>
+      <c r="A58" s="44" t="inlineStr">
+        <is>
+          <t>□ Dev担当が黄色い案件（ローリングス/豊商事/イシダ等）の担当を決めて白にする</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="33" t="inlineStr">
-        <is>
-          <t>担当</t>
-        </is>
-      </c>
-      <c r="B59" s="33" t="inlineStr">
-        <is>
-          <t>今期の仕事</t>
-        </is>
-      </c>
-      <c r="C59" s="33" t="inlineStr">
-        <is>
-          <t>リスク / コメント</t>
+      <c r="A59" s="44" t="inlineStr">
+        <is>
+          <t>□ 東洋捺染Dev（月4人×来期）のフェーズ分割／専用チームを検討</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="43" t="inlineStr">
-        <is>
-          <t>川手</t>
-        </is>
-      </c>
-      <c r="B60" s="23" t="inlineStr">
-        <is>
-          <t>ローリングスRD→イシダ/三菱/東洋RD（神鋼RDの可能性）</t>
-        </is>
-      </c>
-      <c r="C60" s="23" t="inlineStr">
-        <is>
-          <t>10〜12月が最大ボトルネック。三菱外しが効く</t>
+      <c r="A60" s="44" t="inlineStr">
+        <is>
+          <t>□ 来期案件を四半期スロット化</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="44" t="inlineStr">
         <is>
+          <t>□ 神鋼商事・アムリードの時期を確定</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="40" t="inlineStr">
+        <is>
+          <t>担当者メモ</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="33" t="inlineStr">
+        <is>
+          <t>担当</t>
+        </is>
+      </c>
+      <c r="B64" s="33" t="inlineStr">
+        <is>
+          <t>今期の仕事</t>
+        </is>
+      </c>
+      <c r="C64" s="33" t="inlineStr">
+        <is>
+          <t>リスク / コメント</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="45" t="inlineStr">
+        <is>
+          <t>川手</t>
+        </is>
+      </c>
+      <c r="B65" s="23" t="inlineStr">
+        <is>
+          <t>ローリングスRD→イシダ/三菱/東洋RD（神鋼の可能性）</t>
+        </is>
+      </c>
+      <c r="C65" s="23" t="inlineStr">
+        <is>
+          <t>10〜12月が最大ボトルネック。三菱外しが効く</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="46" t="inlineStr">
+        <is>
           <t>小園</t>
         </is>
       </c>
-      <c r="B61" s="23" t="inlineStr">
+      <c r="B66" s="23" t="inlineStr">
         <is>
           <t>ローリングスRD→イシダ/三菱RD（東洋からは外れ）</t>
         </is>
       </c>
-      <c r="C61" s="23" t="inlineStr">
+      <c r="C66" s="23" t="inlineStr">
         <is>
           <t>以前より改善。イシダ+三菱で10〜11月はなお逼迫</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="45" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="47" t="inlineStr">
         <is>
           <t>佐久間</t>
         </is>
       </c>
-      <c r="B62" s="23" t="inlineStr">
+      <c r="B67" s="23" t="inlineStr">
         <is>
           <t>東洋捺染RD（10〜12）</t>
         </is>
       </c>
-      <c r="C62" s="23" t="inlineStr">
-        <is>
-          <t>新規投入。余裕あり。東洋Devの受け皿候補</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="23" t="inlineStr">
+      <c r="C67" s="23" t="inlineStr">
+        <is>
+          <t>余裕あり。東洋Devの受け皿候補</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="23" t="inlineStr">
         <is>
           <t>木村・森崎・伊藤</t>
         </is>
       </c>
-      <c r="B63" s="23" t="inlineStr">
-        <is>
-          <t>イワタニDev 8〜9月</t>
-        </is>
-      </c>
-      <c r="C63" s="23" t="inlineStr">
+      <c r="B68" s="23" t="inlineStr">
+        <is>
+          <t>イワタニDev 8〜9月（Dev担当=白＝割当済）</t>
+        </is>
+      </c>
+      <c r="C68" s="23" t="inlineStr">
         <is>
           <t>成立。後半の未割当Devプール候補</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="15" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="48" t="inlineStr">
         <is>
           <t>未割当</t>
         </is>
       </c>
-      <c r="B64" s="23" t="inlineStr">
-        <is>
-          <t>Dev合計≈111.35人月</t>
-        </is>
-      </c>
-      <c r="C64" s="23" t="inlineStr">
+      <c r="B69" s="23" t="inlineStr">
+        <is>
+          <t>Dev合計≈111.35人月（Dev担当=黄）</t>
+        </is>
+      </c>
+      <c r="C69" s="23" t="inlineStr">
         <is>
           <t>来期リソース計画が本丸</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="18">
     <mergeCell ref="A2:V2"/>
-    <mergeCell ref="A56:H56"/>
+    <mergeCell ref="A44:J44"/>
     <mergeCell ref="B5:N5"/>
     <mergeCell ref="A10:V10"/>
     <mergeCell ref="A28:V28"/>
-    <mergeCell ref="A53:H53"/>
-    <mergeCell ref="A55:H55"/>
-    <mergeCell ref="A44:V44"/>
+    <mergeCell ref="A49:V49"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="A57:H57"/>
     <mergeCell ref="A1:V1"/>
-    <mergeCell ref="A54:H54"/>
-    <mergeCell ref="A52:H52"/>
     <mergeCell ref="A29:N29"/>
+    <mergeCell ref="A60:H60"/>
     <mergeCell ref="A9:V9"/>
     <mergeCell ref="E26:F26"/>
+    <mergeCell ref="A61:H61"/>
     <mergeCell ref="B7:N7"/>
     <mergeCell ref="B6:N6"/>
     <mergeCell ref="A4:V4"/>
+    <mergeCell ref="A58:H58"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Show only ? for uncertain timing bands on gantt
- Remove monthly headcount from TBD/来期 gray cells
- Keep people/month on dated R/D bands; MM stays in left columns

Co-authored-by: kozonoflight <kozonoflight@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/knowledge/人積み/2026-2027_案件人積み.xlsx
+++ b/knowledge/人積み/2026-2027_案件人積み.xlsx
@@ -89,8 +89,8 @@
     <font>
       <name val="Yu Gothic"/>
       <b val="1"/>
-      <color rgb="00333333"/>
-      <sz val="7"/>
+      <color rgb="00555555"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Yu Gothic"/>
@@ -748,7 +748,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ガント数字=その月に必要な人数（人月÷月数）。R=要件定義 / D=開発。Dev担当が白=割当済・黄=未割当。灰帯=時期未定。</t>
+          <t>ガント数字=その月の必要人数（人月÷月数）。R=要件定義 / D=開発。時期未定は「？」。Dev担当: 白=割当済 / 黄=未割当。工数は左列を参照。</t>
         </is>
       </c>
     </row>
@@ -791,21 +791,21 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Dev担当が黄色い案件は未割当。ローリングス/豊商事/イシダDev等の担当決めが必要</t>
+          <t>Dev担当が黄色い案件は未割当。時期未定（？）の工数は左のRD/Dev工数列を見て別途スロット化</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>② 簡易ガント（セル内の数字＝その月に必要な人数）</t>
+          <t>② 簡易ガント（セル内の数字＝その月に必要な人数／時期未定は？）</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>凡例: R=要件定義(青) / D=開発(緑) / 灰=時期未定の開発or混合。数字は必要人数/月。Dev担当列: 白=割当完了 / 黄=未割当</t>
+          <t>凡例: R=要件定義(青) / D=開発(緑) / ？=時期未定(灰)。必要人数は時期が決まっている帯のみ。工数(人月)は左列。Dev担当: 白=割当完了 / 黄=未割当</t>
         </is>
       </c>
     </row>
@@ -1251,62 +1251,52 @@
       <c r="N16" s="17" t="inlineStr"/>
       <c r="O16" s="25" t="inlineStr">
         <is>
-          <t>D
-1人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="P16" s="25" t="inlineStr">
         <is>
-          <t>D
-1人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="Q16" s="25" t="inlineStr">
         <is>
-          <t>D
-1人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="R16" s="25" t="inlineStr">
         <is>
-          <t>D
-1人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="S16" s="25" t="inlineStr">
         <is>
-          <t>D
-1人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="T16" s="25" t="inlineStr">
         <is>
-          <t>D
-1人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="U16" s="25" t="inlineStr">
         <is>
-          <t>D
-1人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="V16" s="25" t="inlineStr">
         <is>
-          <t>D
-1人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="W16" s="25" t="inlineStr">
         <is>
-          <t>D
-1人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="X16" s="25" t="inlineStr">
         <is>
-          <t>D
-1人</t>
+          <t>？</t>
         </is>
       </c>
     </row>
@@ -1362,62 +1352,52 @@
       <c r="N17" s="17" t="inlineStr"/>
       <c r="O17" s="25" t="inlineStr">
         <is>
-          <t>D
-4人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="P17" s="25" t="inlineStr">
         <is>
-          <t>D
-4人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="Q17" s="25" t="inlineStr">
         <is>
-          <t>D
-4人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="R17" s="25" t="inlineStr">
         <is>
-          <t>D
-4人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="S17" s="25" t="inlineStr">
         <is>
-          <t>D
-4人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="T17" s="25" t="inlineStr">
         <is>
-          <t>D
-4人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="U17" s="25" t="inlineStr">
         <is>
-          <t>D
-4人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="V17" s="25" t="inlineStr">
         <is>
-          <t>D
-4人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="W17" s="25" t="inlineStr">
         <is>
-          <t>D
-4人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="X17" s="25" t="inlineStr">
         <is>
-          <t>D
-4人</t>
+          <t>？</t>
         </is>
       </c>
     </row>
@@ -1450,50 +1430,42 @@
       </c>
       <c r="G18" s="25" t="inlineStr">
         <is>
-          <t>?
-1.4人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="H18" s="25" t="inlineStr">
         <is>
-          <t>?
-1.4人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="I18" s="25" t="inlineStr">
         <is>
-          <t>?
-1.4人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="J18" s="25" t="inlineStr">
         <is>
-          <t>?
-1.4人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="K18" s="25" t="inlineStr">
         <is>
-          <t>?
-1.4人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="L18" s="25" t="inlineStr">
         <is>
-          <t>?
-1.4人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="M18" s="25" t="inlineStr">
         <is>
-          <t>?
-1.4人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="N18" s="25" t="inlineStr">
         <is>
-          <t>?
-1.4人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="O18" s="20" t="inlineStr"/>
@@ -1536,50 +1508,42 @@
       </c>
       <c r="G19" s="25" t="inlineStr">
         <is>
-          <t>?
-0.6人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="H19" s="25" t="inlineStr">
         <is>
-          <t>?
-0.6人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="I19" s="25" t="inlineStr">
         <is>
-          <t>?
-0.6人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="J19" s="25" t="inlineStr">
         <is>
-          <t>?
-0.6人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="K19" s="25" t="inlineStr">
         <is>
-          <t>?
-0.6人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="L19" s="25" t="inlineStr">
         <is>
-          <t>?
-0.6人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="M19" s="25" t="inlineStr">
         <is>
-          <t>?
-0.6人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="N19" s="25" t="inlineStr">
         <is>
-          <t>?
-0.6人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="O19" s="20" t="inlineStr"/>
@@ -1630,62 +1594,52 @@
       <c r="N20" s="17" t="inlineStr"/>
       <c r="O20" s="25" t="inlineStr">
         <is>
-          <t>?
-1.3人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="P20" s="25" t="inlineStr">
         <is>
-          <t>?
-1.3人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="Q20" s="25" t="inlineStr">
         <is>
-          <t>?
-1.3人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="R20" s="25" t="inlineStr">
         <is>
-          <t>?
-1.3人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="S20" s="25" t="inlineStr">
         <is>
-          <t>?
-1.3人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="T20" s="25" t="inlineStr">
         <is>
-          <t>?
-1.3人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="U20" s="25" t="inlineStr">
         <is>
-          <t>?
-1.3人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="V20" s="25" t="inlineStr">
         <is>
-          <t>?
-1.3人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="W20" s="25" t="inlineStr">
         <is>
-          <t>?
-1.3人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="X20" s="25" t="inlineStr">
         <is>
-          <t>?
-1.3人</t>
+          <t>？</t>
         </is>
       </c>
     </row>
@@ -1728,62 +1682,52 @@
       <c r="N21" s="17" t="inlineStr"/>
       <c r="O21" s="25" t="inlineStr">
         <is>
-          <t>D
-0.9人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="P21" s="25" t="inlineStr">
         <is>
-          <t>D
-0.9人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="Q21" s="25" t="inlineStr">
         <is>
-          <t>D
-0.9人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="R21" s="25" t="inlineStr">
         <is>
-          <t>D
-0.9人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="S21" s="25" t="inlineStr">
         <is>
-          <t>D
-0.9人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="T21" s="25" t="inlineStr">
         <is>
-          <t>D
-0.9人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="U21" s="25" t="inlineStr">
         <is>
-          <t>D
-0.9人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="V21" s="25" t="inlineStr">
         <is>
-          <t>D
-0.9人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="W21" s="25" t="inlineStr">
         <is>
-          <t>D
-0.9人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="X21" s="25" t="inlineStr">
         <is>
-          <t>D
-0.9人</t>
+          <t>？</t>
         </is>
       </c>
     </row>
@@ -1826,62 +1770,52 @@
       <c r="N22" s="17" t="inlineStr"/>
       <c r="O22" s="25" t="inlineStr">
         <is>
-          <t>D
-0.9人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="P22" s="25" t="inlineStr">
         <is>
-          <t>D
-0.9人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="Q22" s="25" t="inlineStr">
         <is>
-          <t>D
-0.9人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="R22" s="25" t="inlineStr">
         <is>
-          <t>D
-0.9人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="S22" s="25" t="inlineStr">
         <is>
-          <t>D
-0.9人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="T22" s="25" t="inlineStr">
         <is>
-          <t>D
-0.9人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="U22" s="25" t="inlineStr">
         <is>
-          <t>D
-0.9人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="V22" s="25" t="inlineStr">
         <is>
-          <t>D
-0.9人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="W22" s="25" t="inlineStr">
         <is>
-          <t>D
-0.9人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="X22" s="25" t="inlineStr">
         <is>
-          <t>D
-0.9人</t>
+          <t>？</t>
         </is>
       </c>
     </row>
@@ -1924,62 +1858,52 @@
       <c r="N23" s="17" t="inlineStr"/>
       <c r="O23" s="25" t="inlineStr">
         <is>
-          <t>D
-0.5人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="P23" s="25" t="inlineStr">
         <is>
-          <t>D
-0.5人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="Q23" s="25" t="inlineStr">
         <is>
-          <t>D
-0.5人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="R23" s="25" t="inlineStr">
         <is>
-          <t>D
-0.5人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="S23" s="25" t="inlineStr">
         <is>
-          <t>D
-0.5人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="T23" s="25" t="inlineStr">
         <is>
-          <t>D
-0.5人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="U23" s="25" t="inlineStr">
         <is>
-          <t>D
-0.5人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="V23" s="25" t="inlineStr">
         <is>
-          <t>D
-0.5人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="W23" s="25" t="inlineStr">
         <is>
-          <t>D
-0.5人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="X23" s="25" t="inlineStr">
         <is>
-          <t>D
-0.5人</t>
+          <t>？</t>
         </is>
       </c>
     </row>
@@ -2022,62 +1946,52 @@
       <c r="N24" s="17" t="inlineStr"/>
       <c r="O24" s="25" t="inlineStr">
         <is>
-          <t>D
-0.2人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="P24" s="25" t="inlineStr">
         <is>
-          <t>D
-0.2人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="Q24" s="25" t="inlineStr">
         <is>
-          <t>D
-0.2人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="R24" s="25" t="inlineStr">
         <is>
-          <t>D
-0.2人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="S24" s="25" t="inlineStr">
         <is>
-          <t>D
-0.2人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="T24" s="25" t="inlineStr">
         <is>
-          <t>D
-0.2人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="U24" s="25" t="inlineStr">
         <is>
-          <t>D
-0.2人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="V24" s="25" t="inlineStr">
         <is>
-          <t>D
-0.2人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="W24" s="25" t="inlineStr">
         <is>
-          <t>D
-0.2人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="X24" s="25" t="inlineStr">
         <is>
-          <t>D
-0.2人</t>
+          <t>？</t>
         </is>
       </c>
     </row>
@@ -2120,62 +2034,52 @@
       <c r="N25" s="17" t="inlineStr"/>
       <c r="O25" s="25" t="inlineStr">
         <is>
-          <t>D
-0.1人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="P25" s="25" t="inlineStr">
         <is>
-          <t>D
-0.1人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="Q25" s="25" t="inlineStr">
         <is>
-          <t>D
-0.1人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="R25" s="25" t="inlineStr">
         <is>
-          <t>D
-0.1人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="S25" s="25" t="inlineStr">
         <is>
-          <t>D
-0.1人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="T25" s="25" t="inlineStr">
         <is>
-          <t>D
-0.1人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="U25" s="25" t="inlineStr">
         <is>
-          <t>D
-0.1人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="V25" s="25" t="inlineStr">
         <is>
-          <t>D
-0.1人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="W25" s="25" t="inlineStr">
         <is>
-          <t>D
-0.1人</t>
+          <t>？</t>
         </is>
       </c>
       <c r="X25" s="25" t="inlineStr">
         <is>
-          <t>D
-0.1人</t>
+          <t>？</t>
         </is>
       </c>
     </row>
@@ -2202,7 +2106,7 @@
       </c>
       <c r="E26" s="31" t="inlineStr">
         <is>
-          <t>Dev人月合計。ガントの人数=工数÷月数。黄のDev担当=未割当</t>
+          <t>Dev人月合計。？帯の工数は左列参照。黄のDev担当=未割当</t>
         </is>
       </c>
       <c r="G26" s="32" t="n"/>
@@ -2606,7 +2510,7 @@
     <row r="44">
       <c r="A44" s="40" t="inlineStr">
         <is>
-          <t>月別・必要人数合計（全案件・時期が載っている帯のみ。灰の来期は参考）</t>
+          <t>月別・必要人数合計（時期が決まっている帯のみ。？は含めない）</t>
         </is>
       </c>
     </row>
@@ -2707,71 +2611,91 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="20" customHeight="1">
+    <row r="46">
       <c r="A46" s="27" t="inlineStr">
         <is>
           <t>合計(人)</t>
         </is>
       </c>
-      <c r="B46" s="4" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="C46" s="4" t="n">
-        <v>5.3</v>
+      <c r="B46" s="35" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="C46" s="43" t="n">
+        <v>3.3</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>8.1</v>
+        <v>6.1</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>8.1</v>
+        <v>6.1</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>7.1</v>
-      </c>
-      <c r="G46" s="43" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="H46" s="43" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="I46" s="43" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="J46" s="4" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="K46" s="4" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="L46" s="4" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="M46" s="4" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="N46" s="4" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="O46" s="4" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="P46" s="4" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="Q46" s="4" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="R46" s="4" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="S46" s="4" t="n">
-        <v>8.9</v>
+        <v>5.1</v>
+      </c>
+      <c r="G46" s="35" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H46" s="35" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I46" s="35" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J46" s="36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K46" s="36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L46" s="36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M46" s="36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N46" s="36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O46" s="36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P46" s="36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q46" s="36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R46" s="36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S46" s="36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>※上段ガントの各セル人数を月ごとに合算。同じ月に複数案件が重なると必要な延べ人数。</t>
+          <t>※？帯は月按分しない。工数は左のRD工数/Dev工数列を見てスロット化する。</t>
         </is>
       </c>
     </row>
@@ -2898,7 +2822,7 @@
       </c>
       <c r="B54" s="23" t="inlineStr">
         <is>
-          <t>高圧ガス等RDを四半期割</t>
+          <t>？案件のスロット化</t>
         </is>
       </c>
       <c r="C54" s="23" t="inlineStr">
@@ -2934,21 +2858,21 @@
     <row r="58">
       <c r="A58" s="44" t="inlineStr">
         <is>
-          <t>□ Dev担当が黄色い案件（ローリングス/豊商事/イシダ等）の担当を決めて白にする</t>
+          <t>□ Dev担当が黄色い案件の担当を決めて白にする</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="44" t="inlineStr">
         <is>
-          <t>□ 東洋捺染Dev（月4人×来期）のフェーズ分割／専用チームを検討</t>
+          <t>□ ？帯（時期未定）の案件を四半期スロット化（工数は左列）</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="44" t="inlineStr">
         <is>
-          <t>□ 来期案件を四半期スロット化</t>
+          <t>□ 東洋捺染Dev 40人月のフェーズ分割／専用チームを検討</t>
         </is>
       </c>
     </row>

</xml_diff>